<commit_message>
Remove arquivos temporarios da entrega e padroniza tema das metricas
</commit_message>
<xml_diff>
--- a/4992220_Metricas_Qualidade.xlsx
+++ b/4992220_Metricas_Qualidade.xlsx
@@ -146,9 +146,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="ChatGPT">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Raizes do Nordeste">
   <a:themeElements>
-    <a:clrScheme name="ChatGPT">
+    <a:clrScheme name="Raizes do Nordeste">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -198,7 +198,7 @@
         <a:cs typeface="Calibri"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="ChatGPT">
+    <a:fmtScheme name="Raizes do Nordeste">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>

</xml_diff>

<commit_message>
Consolida revisao completa, 72 testes e entrega academica validada
</commit_message>
<xml_diff>
--- a/4992220_Metricas_Qualidade.xlsx
+++ b/4992220_Metricas_Qualidade.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Indicadores" sheetId="1" r:id="Rb6658480024647da"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Testes" sheetId="2" r:id="Raeb9d3f53a5a4a16"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Carga" sheetId="3" r:id="R255b10aea7f44ed3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Indicadores" sheetId="1" r:id="R32a5072e90074304"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Testes" sheetId="2" r:id="Redb81ccbe8cb4844"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Carga" sheetId="3" r:id="Rdfd2f6272f054cc4"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -372,7 +372,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="2" t="str">
-        <x:v>Diego Monteiro de Farias · RU 4992220 · execução local em 24/09/2026</x:v>
+        <x:v>Diego Monteiro de Farias · RU 4992220 · execução local em 28/09/2026</x:v>
       </x:c>
       <x:c r="B3" s="2"/>
       <x:c r="C3" s="2"/>
@@ -468,7 +468,7 @@
       </x:c>
       <x:c r="B8" s="13" t="n">
         <x:f>AVERAGE(Carga!B6:B205)</x:f>
-        <x:v>58.867425000000004</x:v>
+        <x:v>61.120855000000034</x:v>
       </x:c>
       <x:c r="C8" s="11" t="str">
         <x:v>ms</x:v>
@@ -611,14 +611,14 @@
         <x:v>Testes aprovados</x:v>
       </x:c>
       <x:c r="B16" s="2" t="n">
-        <x:f>COUNTIF(Testes!C6:C75,"APROVADO")</x:f>
-        <x:v>70</x:v>
+        <x:f>COUNTIF(Testes!C6:C77,"APROVADO")</x:f>
+        <x:v>72</x:v>
       </x:c>
       <x:c r="C16" s="2" t="str">
         <x:v>casos</x:v>
       </x:c>
       <x:c r="D16" s="2" t="str">
-        <x:v>52 Python e 18 navegador</x:v>
+        <x:v>54 Python e 18 navegador</x:v>
       </x:c>
       <x:c r="E16" s="2"/>
       <x:c r="F16" s="2"/>
@@ -630,7 +630,7 @@
         <x:v>P95 da resposta</x:v>
       </x:c>
       <x:c r="B17" s="8" t="n">
-        <x:v>208.004</x:v>
+        <x:v>149.676</x:v>
       </x:c>
       <x:c r="C17" s="2" t="str">
         <x:v>ms</x:v>
@@ -739,7 +739,7 @@
         <x:v>versão</x:v>
       </x:c>
       <x:c r="D24" s="11" t="str">
-        <x:v>Revisão local v0.4</x:v>
+        <x:v>Revisão local v0.5</x:v>
       </x:c>
       <x:c r="E24" s="2"/>
       <x:c r="F24" s="2"/>
@@ -2961,7 +2961,7 @@
         <x:v>APROVADO</x:v>
       </x:c>
       <x:c r="D6" s="8" t="n">
-        <x:v>594.193</x:v>
+        <x:v>1140.176</x:v>
       </x:c>
       <x:c r="E6" s="2"/>
       <x:c r="F6" s="2"/>
@@ -2979,7 +2979,7 @@
         <x:v>APROVADO</x:v>
       </x:c>
       <x:c r="D7" s="8" t="n">
-        <x:v>462.797</x:v>
+        <x:v>795.569</x:v>
       </x:c>
       <x:c r="E7" s="2"/>
       <x:c r="F7" s="2"/>
@@ -2997,7 +2997,7 @@
         <x:v>APROVADO</x:v>
       </x:c>
       <x:c r="D8" s="8" t="n">
-        <x:v>4.383</x:v>
+        <x:v>3.288</x:v>
       </x:c>
       <x:c r="E8" s="2"/>
       <x:c r="F8" s="2"/>
@@ -3015,7 +3015,7 @@
         <x:v>APROVADO</x:v>
       </x:c>
       <x:c r="D9" s="8" t="n">
-        <x:v>585.628</x:v>
+        <x:v>613.481</x:v>
       </x:c>
       <x:c r="E9" s="2"/>
       <x:c r="F9" s="2"/>
@@ -3033,7 +3033,7 @@
         <x:v>APROVADO</x:v>
       </x:c>
       <x:c r="D10" s="8" t="n">
-        <x:v>562.718</x:v>
+        <x:v>571.874</x:v>
       </x:c>
       <x:c r="E10" s="2"/>
       <x:c r="F10" s="2"/>
@@ -3051,7 +3051,7 @@
         <x:v>APROVADO</x:v>
       </x:c>
       <x:c r="D11" s="8" t="n">
-        <x:v>525.331</x:v>
+        <x:v>526.794</x:v>
       </x:c>
       <x:c r="E11" s="2"/>
       <x:c r="F11" s="2"/>
@@ -3069,7 +3069,7 @@
         <x:v>APROVADO</x:v>
       </x:c>
       <x:c r="D12" s="8" t="n">
-        <x:v>515.63</x:v>
+        <x:v>529.557</x:v>
       </x:c>
       <x:c r="E12" s="2"/>
       <x:c r="F12" s="2"/>
@@ -3087,7 +3087,7 @@
         <x:v>APROVADO</x:v>
       </x:c>
       <x:c r="D13" s="8" t="n">
-        <x:v>529.149</x:v>
+        <x:v>527.175</x:v>
       </x:c>
       <x:c r="E13" s="2"/>
       <x:c r="F13" s="2"/>
@@ -3105,7 +3105,7 @@
         <x:v>APROVADO</x:v>
       </x:c>
       <x:c r="D14" s="8" t="n">
-        <x:v>530.112</x:v>
+        <x:v>526.238</x:v>
       </x:c>
       <x:c r="E14" s="2"/>
       <x:c r="F14" s="2"/>
@@ -3123,7 +3123,7 @@
         <x:v>APROVADO</x:v>
       </x:c>
       <x:c r="D15" s="8" t="n">
-        <x:v>529.396</x:v>
+        <x:v>528.914</x:v>
       </x:c>
       <x:c r="E15" s="2"/>
       <x:c r="F15" s="2"/>
@@ -3141,7 +3141,7 @@
         <x:v>APROVADO</x:v>
       </x:c>
       <x:c r="D16" s="8" t="n">
-        <x:v>603.68</x:v>
+        <x:v>571.239</x:v>
       </x:c>
       <x:c r="E16" s="2"/>
       <x:c r="F16" s="2"/>
@@ -3159,7 +3159,7 @@
         <x:v>APROVADO</x:v>
       </x:c>
       <x:c r="D17" s="8" t="n">
-        <x:v>560.774</x:v>
+        <x:v>576.187</x:v>
       </x:c>
       <x:c r="E17" s="2"/>
       <x:c r="F17" s="2"/>
@@ -3168,16 +3168,16 @@
     </x:row>
     <x:row r="18" ht="36" customHeight="1">
       <x:c r="A18" s="2" t="str">
-        <x:v>RG01</x:v>
+        <x:v>API09</x:v>
       </x:c>
       <x:c r="B18" s="11" t="str">
-        <x:v>Credencial não ASCII retorna 401 e preserva a execução do servidor.</x:v>
+        <x:v>Cliente desconectado após commit não provoca segunda resposta nem duplica efeitos ao repetir.</x:v>
       </x:c>
       <x:c r="C18" s="2" t="str">
         <x:v>APROVADO</x:v>
       </x:c>
       <x:c r="D18" s="8" t="n">
-        <x:v>524.065</x:v>
+        <x:v>541.147</x:v>
       </x:c>
       <x:c r="E18" s="2"/>
       <x:c r="F18" s="2"/>
@@ -3186,16 +3186,16 @@
     </x:row>
     <x:row r="19" ht="36" customHeight="1">
       <x:c r="A19" s="2" t="str">
-        <x:v>RG04</x:v>
+        <x:v>API10</x:v>
       </x:c>
       <x:c r="B19" s="11" t="str">
-        <x:v>Segunda instância na mesma porta é recusada e a primeira continua saudável.</x:v>
+        <x:v>Corpo menor que Content-Length retorna 400 sem criar pedido, mesmo com JSON válido.</x:v>
       </x:c>
       <x:c r="C19" s="2" t="str">
         <x:v>APROVADO</x:v>
       </x:c>
       <x:c r="D19" s="8" t="n">
-        <x:v>525.211</x:v>
+        <x:v>528.964</x:v>
       </x:c>
       <x:c r="E19" s="2"/>
       <x:c r="F19" s="2"/>
@@ -3204,16 +3204,16 @@
     </x:row>
     <x:row r="20" ht="36" customHeight="1">
       <x:c r="A20" s="2" t="str">
-        <x:v>PR01</x:v>
+        <x:v>RG01</x:v>
       </x:c>
       <x:c r="B20" s="11" t="str">
-        <x:v>Aprovar pendência reduz estoque e soma pontos uma vez; consulta recupera os itens.</x:v>
+        <x:v>Credencial não ASCII retorna 401 e preserva a execução do servidor.</x:v>
       </x:c>
       <x:c r="C20" s="2" t="str">
         <x:v>APROVADO</x:v>
       </x:c>
       <x:c r="D20" s="8" t="n">
-        <x:v>35.524</x:v>
+        <x:v>531.597</x:v>
       </x:c>
       <x:c r="E20" s="2"/>
       <x:c r="F20" s="2"/>
@@ -3222,16 +3222,16 @@
     </x:row>
     <x:row r="21" ht="36" customHeight="1">
       <x:c r="A21" s="2" t="str">
-        <x:v>PR02</x:v>
+        <x:v>RG04</x:v>
       </x:c>
       <x:c r="B21" s="11" t="str">
-        <x:v>Recusar pendência e repetir a recusa preserva estoque e pontos.</x:v>
+        <x:v>Segunda instância na mesma porta é recusada e a primeira continua saudável.</x:v>
       </x:c>
       <x:c r="C21" s="2" t="str">
         <x:v>APROVADO</x:v>
       </x:c>
       <x:c r="D21" s="8" t="n">
-        <x:v>28.343</x:v>
+        <x:v>530.397</x:v>
       </x:c>
       <x:c r="E21" s="2"/>
       <x:c r="F21" s="2"/>
@@ -3240,16 +3240,16 @@
     </x:row>
     <x:row r="22" ht="36" customHeight="1">
       <x:c r="A22" s="2" t="str">
-        <x:v>PR03</x:v>
+        <x:v>PR01</x:v>
       </x:c>
       <x:c r="B22" s="11" t="str">
-        <x:v>Uma decisão terminal não pode ser invertida, inclusive em pedidos sem pendência.</x:v>
+        <x:v>Aprovar pendência reduz estoque e soma pontos uma vez; consulta recupera os itens.</x:v>
       </x:c>
       <x:c r="C22" s="2" t="str">
         <x:v>APROVADO</x:v>
       </x:c>
       <x:c r="D22" s="8" t="n">
-        <x:v>31.006</x:v>
+        <x:v>46.204</x:v>
       </x:c>
       <x:c r="E22" s="2"/>
       <x:c r="F22" s="2"/>
@@ -3258,16 +3258,16 @@
     </x:row>
     <x:row r="23" ht="36" customHeight="1">
       <x:c r="A23" s="2" t="str">
-        <x:v>PR04</x:v>
+        <x:v>PR02</x:v>
       </x:c>
       <x:c r="B23" s="11" t="str">
-        <x:v>Vinte aprovações simultâneas da mesma pendência têm um único efeito.</x:v>
+        <x:v>Recusar pendência e repetir a recusa preserva estoque e pontos.</x:v>
       </x:c>
       <x:c r="C23" s="2" t="str">
         <x:v>APROVADO</x:v>
       </x:c>
       <x:c r="D23" s="8" t="n">
-        <x:v>191.831</x:v>
+        <x:v>37.512</x:v>
       </x:c>
       <x:c r="E23" s="2"/>
       <x:c r="F23" s="2"/>
@@ -3276,16 +3276,16 @@
     </x:row>
     <x:row r="24" ht="36" customHeight="1">
       <x:c r="A24" s="2" t="str">
-        <x:v>PR05</x:v>
+        <x:v>PR03</x:v>
       </x:c>
       <x:c r="B24" s="11" t="str">
-        <x:v>Aprovação e recusa concorrentes encerram a pendência com uma única decisão.</x:v>
+        <x:v>Uma decisão terminal não pode ser invertida, inclusive em pedidos sem pendência.</x:v>
       </x:c>
       <x:c r="C24" s="2" t="str">
         <x:v>APROVADO</x:v>
       </x:c>
       <x:c r="D24" s="8" t="n">
-        <x:v>30.553</x:v>
+        <x:v>42.939</x:v>
       </x:c>
       <x:c r="E24" s="2"/>
       <x:c r="F24" s="2"/>
@@ -3294,16 +3294,16 @@
     </x:row>
     <x:row r="25" ht="36" customHeight="1">
       <x:c r="A25" s="2" t="str">
-        <x:v>PR06</x:v>
+        <x:v>PR04</x:v>
       </x:c>
       <x:c r="B25" s="11" t="str">
-        <x:v>Duas pendências disputam as últimas dez unidades sem venda acima do estoque.</x:v>
+        <x:v>Vinte aprovações simultâneas da mesma pendência têm um único efeito.</x:v>
       </x:c>
       <x:c r="C25" s="2" t="str">
         <x:v>APROVADO</x:v>
       </x:c>
       <x:c r="D25" s="8" t="n">
-        <x:v>47.265</x:v>
+        <x:v>244.749</x:v>
       </x:c>
       <x:c r="E25" s="2"/>
       <x:c r="F25" s="2"/>
@@ -3312,16 +3312,16 @@
     </x:row>
     <x:row r="26" ht="36" customHeight="1">
       <x:c r="A26" s="2" t="str">
-        <x:v>PR07</x:v>
+        <x:v>PR05</x:v>
       </x:c>
       <x:c r="B26" s="11" t="str">
-        <x:v>Falta de estoque mantém pendência sem baixa parcial e permite recusa posterior.</x:v>
+        <x:v>Aprovação e recusa concorrentes encerram a pendência com uma única decisão.</x:v>
       </x:c>
       <x:c r="C26" s="2" t="str">
         <x:v>APROVADO</x:v>
       </x:c>
       <x:c r="D26" s="8" t="n">
-        <x:v>34.911</x:v>
+        <x:v>44.265</x:v>
       </x:c>
       <x:c r="E26" s="2"/>
       <x:c r="F26" s="2"/>
@@ -3330,16 +3330,16 @@
     </x:row>
     <x:row r="27" ht="36" customHeight="1">
       <x:c r="A27" s="2" t="str">
-        <x:v>PR08</x:v>
+        <x:v>PR06</x:v>
       </x:c>
       <x:c r="B27" s="11" t="str">
-        <x:v>Somente o proprietário confere a pendência; pedido inexistente retorna 404.</x:v>
+        <x:v>Duas pendências disputam as últimas dez unidades sem venda acima do estoque.</x:v>
       </x:c>
       <x:c r="C27" s="2" t="str">
         <x:v>APROVADO</x:v>
       </x:c>
       <x:c r="D27" s="8" t="n">
-        <x:v>24.519</x:v>
+        <x:v>46.384</x:v>
       </x:c>
       <x:c r="E27" s="2"/>
       <x:c r="F27" s="2"/>
@@ -3348,16 +3348,16 @@
     </x:row>
     <x:row r="28" ht="36" customHeight="1">
       <x:c r="A28" s="2" t="str">
-        <x:v>PR09</x:v>
+        <x:v>PR07</x:v>
       </x:c>
       <x:c r="B28" s="11" t="str">
-        <x:v>A conferência aceita apenas o campo payment com approved ou declined.</x:v>
+        <x:v>Falta de estoque mantém pendência sem baixa parcial e permite recusa posterior.</x:v>
       </x:c>
       <x:c r="C28" s="2" t="str">
         <x:v>APROVADO</x:v>
       </x:c>
       <x:c r="D28" s="8" t="n">
-        <x:v>22.207</x:v>
+        <x:v>47.744</x:v>
       </x:c>
       <x:c r="E28" s="2"/>
       <x:c r="F28" s="2"/>
@@ -3366,16 +3366,16 @@
     </x:row>
     <x:row r="29" ht="36" customHeight="1">
       <x:c r="A29" s="2" t="str">
-        <x:v>PR10</x:v>
+        <x:v>PR08</x:v>
       </x:c>
       <x:c r="B29" s="11" t="str">
-        <x:v>Migração preserva dados; pendência antiga permite recusa e impede aprovação sem itens salvos.</x:v>
+        <x:v>Somente o proprietário confere a pendência; pedido inexistente retorna 404.</x:v>
       </x:c>
       <x:c r="C29" s="2" t="str">
         <x:v>APROVADO</x:v>
       </x:c>
       <x:c r="D29" s="8" t="n">
-        <x:v>53.82</x:v>
+        <x:v>29.956</x:v>
       </x:c>
       <x:c r="E29" s="2"/>
       <x:c r="F29" s="2"/>
@@ -3384,16 +3384,16 @@
     </x:row>
     <x:row r="30" ht="36" customHeight="1">
       <x:c r="A30" s="2" t="str">
-        <x:v>PR11</x:v>
+        <x:v>PR09</x:v>
       </x:c>
       <x:c r="B30" s="11" t="str">
-        <x:v>Reinício recupera pendência de João Pessoa e aprova sem pontos quando a fidelidade está desmarcada.</x:v>
+        <x:v>A conferência aceita apenas o campo payment com approved ou declined.</x:v>
       </x:c>
       <x:c r="C30" s="2" t="str">
         <x:v>APROVADO</x:v>
       </x:c>
       <x:c r="D30" s="8" t="n">
-        <x:v>29.394</x:v>
+        <x:v>29.019</x:v>
       </x:c>
       <x:c r="E30" s="2"/>
       <x:c r="F30" s="2"/>
@@ -3402,16 +3402,16 @@
     </x:row>
     <x:row r="31" ht="36" customHeight="1">
       <x:c r="A31" s="2" t="str">
-        <x:v>PR12</x:v>
+        <x:v>PR10</x:v>
       </x:c>
       <x:c r="B31" s="11" t="str">
-        <x:v>Falha ao registrar a transição desfaz estoque, pontos e estado; nova tentativa pode concluir.</x:v>
+        <x:v>Migração preserva dados; pendência antiga permite recusa e impede aprovação sem itens salvos.</x:v>
       </x:c>
       <x:c r="C31" s="2" t="str">
         <x:v>APROVADO</x:v>
       </x:c>
       <x:c r="D31" s="8" t="n">
-        <x:v>38.418</x:v>
+        <x:v>70.521</x:v>
       </x:c>
       <x:c r="E31" s="2"/>
       <x:c r="F31" s="2"/>
@@ -3420,16 +3420,16 @@
     </x:row>
     <x:row r="32" ht="36" customHeight="1">
       <x:c r="A32" s="2" t="str">
-        <x:v>SE01</x:v>
+        <x:v>PR11</x:v>
       </x:c>
       <x:c r="B32" s="11" t="str">
-        <x:v>Outro cliente não acessa pedido alheio.</x:v>
+        <x:v>Reinício recupera pendência de João Pessoa e aprova sem pontos quando a fidelidade está desmarcada.</x:v>
       </x:c>
       <x:c r="C32" s="2" t="str">
         <x:v>APROVADO</x:v>
       </x:c>
       <x:c r="D32" s="8" t="n">
-        <x:v>19.075</x:v>
+        <x:v>33.581</x:v>
       </x:c>
       <x:c r="E32" s="2"/>
       <x:c r="F32" s="2"/>
@@ -3438,16 +3438,16 @@
     </x:row>
     <x:row r="33" ht="36" customHeight="1">
       <x:c r="A33" s="2" t="str">
-        <x:v>SE02</x:v>
+        <x:v>PR12</x:v>
       </x:c>
       <x:c r="B33" s="11" t="str">
-        <x:v>Operador da unidade incorreta recebe 403; unidade correta consulta.</x:v>
+        <x:v>Falha ao registrar a transição desfaz estoque, pontos e estado; nova tentativa pode concluir.</x:v>
       </x:c>
       <x:c r="C33" s="2" t="str">
         <x:v>APROVADO</x:v>
       </x:c>
       <x:c r="D33" s="8" t="n">
-        <x:v>21.209</x:v>
+        <x:v>51.504</x:v>
       </x:c>
       <x:c r="E33" s="2"/>
       <x:c r="F33" s="2"/>
@@ -3456,16 +3456,16 @@
     </x:row>
     <x:row r="34" ht="36" customHeight="1">
       <x:c r="A34" s="2" t="str">
-        <x:v>TS01</x:v>
+        <x:v>SE01</x:v>
       </x:c>
       <x:c r="B34" s="11" t="str">
-        <x:v>Aprovar pedido em APP, WEB, TOTEM, BALCAO e PICKUP.</x:v>
+        <x:v>Outro cliente não acessa pedido alheio.</x:v>
       </x:c>
       <x:c r="C34" s="2" t="str">
         <x:v>APROVADO</x:v>
       </x:c>
       <x:c r="D34" s="8" t="n">
-        <x:v>569.854</x:v>
+        <x:v>28.217</x:v>
       </x:c>
       <x:c r="E34" s="2"/>
       <x:c r="F34" s="2"/>
@@ -3474,16 +3474,16 @@
     </x:row>
     <x:row r="35" ht="36" customHeight="1">
       <x:c r="A35" s="2" t="str">
-        <x:v>TS02</x:v>
+        <x:v>SE02</x:v>
       </x:c>
       <x:c r="B35" s="11" t="str">
-        <x:v>Recusa não altera estoque nem concede pontos.</x:v>
+        <x:v>Operador da unidade incorreta recebe 403; unidade correta consulta.</x:v>
       </x:c>
       <x:c r="C35" s="2" t="str">
         <x:v>APROVADO</x:v>
       </x:c>
       <x:c r="D35" s="8" t="n">
-        <x:v>531.757</x:v>
+        <x:v>24.94</x:v>
       </x:c>
       <x:c r="E35" s="2"/>
       <x:c r="F35" s="2"/>
@@ -3492,16 +3492,16 @@
     </x:row>
     <x:row r="36" ht="36" customHeight="1">
       <x:c r="A36" s="2" t="str">
-        <x:v>TS03</x:v>
+        <x:v>TS01</x:v>
       </x:c>
       <x:c r="B36" s="11" t="str">
-        <x:v>Timeout fica pendente; repetição preserva o mesmo pedido.</x:v>
+        <x:v>Aprovar pedido em APP, WEB, TOTEM, BALCAO e PICKUP.</x:v>
       </x:c>
       <x:c r="C36" s="2" t="str">
         <x:v>APROVADO</x:v>
       </x:c>
       <x:c r="D36" s="8" t="n">
-        <x:v>527.161</x:v>
+        <x:v>558.798</x:v>
       </x:c>
       <x:c r="E36" s="2"/>
       <x:c r="F36" s="2"/>
@@ -3510,16 +3510,16 @@
     </x:row>
     <x:row r="37" ht="36" customHeight="1">
       <x:c r="A37" s="2" t="str">
-        <x:v>TS04</x:v>
+        <x:v>TS02</x:v>
       </x:c>
       <x:c r="B37" s="11" t="str">
-        <x:v>Repetir pedido confirmado gera um pedido, 52 pontos e um evento.</x:v>
+        <x:v>Recusa não altera estoque nem concede pontos.</x:v>
       </x:c>
       <x:c r="C37" s="2" t="str">
         <x:v>APROVADO</x:v>
       </x:c>
       <x:c r="D37" s="8" t="n">
-        <x:v>557.626</x:v>
+        <x:v>531.904</x:v>
       </x:c>
       <x:c r="E37" s="2"/>
       <x:c r="F37" s="2"/>
@@ -3528,16 +3528,16 @@
     </x:row>
     <x:row r="38" ht="36" customHeight="1">
       <x:c r="A38" s="2" t="str">
-        <x:v>TS05</x:v>
+        <x:v>TS03</x:v>
       </x:c>
       <x:c r="B38" s="11" t="str">
-        <x:v>Mesma chave com conteúdo alterado retorna conflito.</x:v>
+        <x:v>Timeout fica pendente; repetição preserva o mesmo pedido.</x:v>
       </x:c>
       <x:c r="C38" s="2" t="str">
         <x:v>APROVADO</x:v>
       </x:c>
       <x:c r="D38" s="8" t="n">
-        <x:v>526.374</x:v>
+        <x:v>529.952</x:v>
       </x:c>
       <x:c r="E38" s="2"/>
       <x:c r="F38" s="2"/>
@@ -3546,16 +3546,16 @@
     </x:row>
     <x:row r="39" ht="36" customHeight="1">
       <x:c r="A39" s="2" t="str">
-        <x:v>TS06</x:v>
+        <x:v>TS04</x:v>
       </x:c>
       <x:c r="B39" s="11" t="str">
-        <x:v>Pedido maior que estoque restante falha sem alteração parcial.</x:v>
+        <x:v>Repetir pedido confirmado gera um pedido, 52 pontos e um evento.</x:v>
       </x:c>
       <x:c r="C39" s="2" t="str">
         <x:v>APROVADO</x:v>
       </x:c>
       <x:c r="D39" s="8" t="n">
-        <x:v>530.367</x:v>
+        <x:v>561.023</x:v>
       </x:c>
       <x:c r="E39" s="2"/>
       <x:c r="F39" s="2"/>
@@ -3564,16 +3564,16 @@
     </x:row>
     <x:row r="40" ht="36" customHeight="1">
       <x:c r="A40" s="2" t="str">
-        <x:v>TS07</x:v>
+        <x:v>TS05</x:v>
       </x:c>
       <x:c r="B40" s="11" t="str">
-        <x:v>Compra em Recife preserva estoque da unidade João Pessoa.</x:v>
+        <x:v>Mesma chave com conteúdo alterado retorna conflito.</x:v>
       </x:c>
       <x:c r="C40" s="2" t="str">
         <x:v>APROVADO</x:v>
       </x:c>
       <x:c r="D40" s="8" t="n">
-        <x:v>528.281</x:v>
+        <x:v>541.486</x:v>
       </x:c>
       <x:c r="E40" s="2"/>
       <x:c r="F40" s="2"/>
@@ -3582,16 +3582,16 @@
     </x:row>
     <x:row r="41" ht="36" customHeight="1">
       <x:c r="A41" s="2" t="str">
-        <x:v>TS08</x:v>
+        <x:v>TS06</x:v>
       </x:c>
       <x:c r="B41" s="11" t="str">
-        <x:v>Compra sem fidelidade confirma com zero pontos.</x:v>
+        <x:v>Pedido maior que estoque restante falha sem alteração parcial.</x:v>
       </x:c>
       <x:c r="C41" s="2" t="str">
         <x:v>APROVADO</x:v>
       </x:c>
       <x:c r="D41" s="8" t="n">
-        <x:v>527.759</x:v>
+        <x:v>528.947</x:v>
       </x:c>
       <x:c r="E41" s="2"/>
       <x:c r="F41" s="2"/>
@@ -3600,16 +3600,16 @@
     </x:row>
     <x:row r="42" ht="36" customHeight="1">
       <x:c r="A42" s="2" t="str">
-        <x:v>TS09</x:v>
+        <x:v>TS07</x:v>
       </x:c>
       <x:c r="B42" s="11" t="str">
-        <x:v>Cupom inexistente não cria pedido nem reduz estoque.</x:v>
+        <x:v>Compra em Recife preserva estoque da unidade João Pessoa.</x:v>
       </x:c>
       <x:c r="C42" s="2" t="str">
         <x:v>APROVADO</x:v>
       </x:c>
       <x:c r="D42" s="8" t="n">
-        <x:v>530.305</x:v>
+        <x:v>527.532</x:v>
       </x:c>
       <x:c r="E42" s="2"/>
       <x:c r="F42" s="2"/>
@@ -3618,16 +3618,16 @@
     </x:row>
     <x:row r="43" ht="36" customHeight="1">
       <x:c r="A43" s="2" t="str">
-        <x:v>TS10</x:v>
+        <x:v>TS08</x:v>
       </x:c>
       <x:c r="B43" s="11" t="str">
-        <x:v>Quantidade zero retorna QUANTIDADE_INVALIDA.</x:v>
+        <x:v>Compra sem fidelidade confirma com zero pontos.</x:v>
       </x:c>
       <x:c r="C43" s="2" t="str">
         <x:v>APROVADO</x:v>
       </x:c>
       <x:c r="D43" s="8" t="n">
-        <x:v>529.126</x:v>
+        <x:v>526.739</x:v>
       </x:c>
       <x:c r="E43" s="2"/>
       <x:c r="F43" s="2"/>
@@ -3636,16 +3636,16 @@
     </x:row>
     <x:row r="44" ht="36" customHeight="1">
       <x:c r="A44" s="2" t="str">
-        <x:v>TS11</x:v>
+        <x:v>TS09</x:v>
       </x:c>
       <x:c r="B44" s="11" t="str">
-        <x:v>Carrinho vazio retorna CARRINHO_INVALIDO.</x:v>
+        <x:v>Cupom inexistente não cria pedido nem reduz estoque.</x:v>
       </x:c>
       <x:c r="C44" s="2" t="str">
         <x:v>APROVADO</x:v>
       </x:c>
       <x:c r="D44" s="8" t="n">
-        <x:v>528.118</x:v>
+        <x:v>526.036</x:v>
       </x:c>
       <x:c r="E44" s="2"/>
       <x:c r="F44" s="2"/>
@@ -3654,16 +3654,16 @@
     </x:row>
     <x:row r="45" ht="36" customHeight="1">
       <x:c r="A45" s="2" t="str">
-        <x:v>TS12</x:v>
+        <x:v>TS10</x:v>
       </x:c>
       <x:c r="B45" s="11" t="str">
-        <x:v>Unidade ou canal desconhecido é rejeitado.</x:v>
+        <x:v>Quantidade zero retorna QUANTIDADE_INVALIDA.</x:v>
       </x:c>
       <x:c r="C45" s="2" t="str">
         <x:v>APROVADO</x:v>
       </x:c>
       <x:c r="D45" s="8" t="n">
-        <x:v>525.115</x:v>
+        <x:v>523.511</x:v>
       </x:c>
       <x:c r="E45" s="2"/>
       <x:c r="F45" s="2"/>
@@ -3672,16 +3672,16 @@
     </x:row>
     <x:row r="46" ht="36" customHeight="1">
       <x:c r="A46" s="2" t="str">
-        <x:v>TS13</x:v>
+        <x:v>TS11</x:v>
       </x:c>
       <x:c r="B46" s="11" t="str">
-        <x:v>Produto inexistente e tentativa de injeção não alteram o banco.</x:v>
+        <x:v>Carrinho vazio retorna CARRINHO_INVALIDO.</x:v>
       </x:c>
       <x:c r="C46" s="2" t="str">
         <x:v>APROVADO</x:v>
       </x:c>
       <x:c r="D46" s="8" t="n">
-        <x:v>525.192</x:v>
+        <x:v>527.865</x:v>
       </x:c>
       <x:c r="E46" s="2"/>
       <x:c r="F46" s="2"/>
@@ -3690,16 +3690,16 @@
     </x:row>
     <x:row r="47" ht="36" customHeight="1">
       <x:c r="A47" s="2" t="str">
-        <x:v>TS14</x:v>
+        <x:v>TS12</x:v>
       </x:c>
       <x:c r="B47" s="11" t="str">
-        <x:v>Nova instância recupera pedido e reconhece sua chave.</x:v>
+        <x:v>Unidade ou canal desconhecido é rejeitado.</x:v>
       </x:c>
       <x:c r="C47" s="2" t="str">
         <x:v>APROVADO</x:v>
       </x:c>
       <x:c r="D47" s="8" t="n">
-        <x:v>527.646</x:v>
+        <x:v>539.884</x:v>
       </x:c>
       <x:c r="E47" s="2"/>
       <x:c r="F47" s="2"/>
@@ -3708,16 +3708,16 @@
     </x:row>
     <x:row r="48" ht="36" customHeight="1">
       <x:c r="A48" s="2" t="str">
-        <x:v>TS15</x:v>
+        <x:v>TS13</x:v>
       </x:c>
       <x:c r="B48" s="11" t="str">
-        <x:v>Fidelidade acumula 104 pontos em duas unidades sem duplicação.</x:v>
+        <x:v>Produto inexistente e tentativa de injeção não alteram o banco.</x:v>
       </x:c>
       <x:c r="C48" s="2" t="str">
         <x:v>APROVADO</x:v>
       </x:c>
       <x:c r="D48" s="8" t="n">
-        <x:v>527.392</x:v>
+        <x:v>526.01</x:v>
       </x:c>
       <x:c r="E48" s="2"/>
       <x:c r="F48" s="2"/>
@@ -3726,16 +3726,16 @@
     </x:row>
     <x:row r="49" ht="36" customHeight="1">
       <x:c r="A49" s="2" t="str">
-        <x:v>TS16</x:v>
+        <x:v>TS14</x:v>
       </x:c>
       <x:c r="B49" s="11" t="str">
-        <x:v>Resposta inválida do gateway desfaz a transação integralmente.</x:v>
+        <x:v>Nova instância recupera pedido e reconhece sua chave.</x:v>
       </x:c>
       <x:c r="C49" s="2" t="str">
         <x:v>APROVADO</x:v>
       </x:c>
       <x:c r="D49" s="8" t="n">
-        <x:v>523.364</x:v>
+        <x:v>527.142</x:v>
       </x:c>
       <x:c r="E49" s="2"/>
       <x:c r="F49" s="2"/>
@@ -3744,16 +3744,16 @@
     </x:row>
     <x:row r="50" ht="36" customHeight="1">
       <x:c r="A50" s="2" t="str">
-        <x:v>TS17</x:v>
+        <x:v>TS15</x:v>
       </x:c>
       <x:c r="B50" s="11" t="str">
-        <x:v>Cada resultado cria um evento sem identificador de cliente ou payload.</x:v>
+        <x:v>Fidelidade acumula 104 pontos em duas unidades sem duplicação.</x:v>
       </x:c>
       <x:c r="C50" s="2" t="str">
         <x:v>APROVADO</x:v>
       </x:c>
       <x:c r="D50" s="8" t="n">
-        <x:v>557.785</x:v>
+        <x:v>542.459</x:v>
       </x:c>
       <x:c r="E50" s="2"/>
       <x:c r="F50" s="2"/>
@@ -3762,16 +3762,16 @@
     </x:row>
     <x:row r="51" ht="36" customHeight="1">
       <x:c r="A51" s="2" t="str">
-        <x:v>TS18</x:v>
+        <x:v>TS16</x:v>
       </x:c>
       <x:c r="B51" s="11" t="str">
-        <x:v>Consultar pedido inexistente retorna 404.</x:v>
+        <x:v>Resposta inválida do gateway desfaz a transação integralmente.</x:v>
       </x:c>
       <x:c r="C51" s="2" t="str">
         <x:v>APROVADO</x:v>
       </x:c>
       <x:c r="D51" s="8" t="n">
-        <x:v>529.406</x:v>
+        <x:v>526.226</x:v>
       </x:c>
       <x:c r="E51" s="2"/>
       <x:c r="F51" s="2"/>
@@ -3780,16 +3780,16 @@
     </x:row>
     <x:row r="52" ht="36" customHeight="1">
       <x:c r="A52" s="2" t="str">
-        <x:v>TU01</x:v>
+        <x:v>TS17</x:v>
       </x:c>
       <x:c r="B52" s="11" t="str">
-        <x:v>Valores exatos: 5800 - 580 = 5220 centavos; 52 pontos.</x:v>
+        <x:v>Cada resultado cria um evento sem identificador de cliente ou payload.</x:v>
       </x:c>
       <x:c r="C52" s="2" t="str">
         <x:v>APROVADO</x:v>
       </x:c>
       <x:c r="D52" s="8" t="n">
-        <x:v>0.107</x:v>
+        <x:v>541.666</x:v>
       </x:c>
       <x:c r="E52" s="2"/>
       <x:c r="F52" s="2"/>
@@ -3798,16 +3798,16 @@
     </x:row>
     <x:row r="53" ht="36" customHeight="1">
       <x:c r="A53" s="2" t="str">
-        <x:v>TU02</x:v>
+        <x:v>TS18</x:v>
       </x:c>
       <x:c r="B53" s="11" t="str">
-        <x:v>Sem cupom e sem fidelidade: total 5800 e zero pontos.</x:v>
+        <x:v>Consultar pedido inexistente retorna 404.</x:v>
       </x:c>
       <x:c r="C53" s="2" t="str">
         <x:v>APROVADO</x:v>
       </x:c>
       <x:c r="D53" s="8" t="n">
-        <x:v>0.059</x:v>
+        <x:v>527.842</x:v>
       </x:c>
       <x:c r="E53" s="2"/>
       <x:c r="F53" s="2"/>
@@ -3816,16 +3816,16 @@
     </x:row>
     <x:row r="54" ht="36" customHeight="1">
       <x:c r="A54" s="2" t="str">
-        <x:v>TU03</x:v>
+        <x:v>TU01</x:v>
       </x:c>
       <x:c r="B54" s="11" t="str">
-        <x:v>Aceitar 1 e 10; rejeitar 0, -1, 11, 1.5, string e booleano.</x:v>
+        <x:v>Valores exatos: 5800 - 580 = 5220 centavos; 52 pontos.</x:v>
       </x:c>
       <x:c r="C54" s="2" t="str">
         <x:v>APROVADO</x:v>
       </x:c>
       <x:c r="D54" s="8" t="n">
-        <x:v>0.185</x:v>
+        <x:v>0.147</x:v>
       </x:c>
       <x:c r="E54" s="2"/>
       <x:c r="F54" s="2"/>
@@ -3834,16 +3834,16 @@
     </x:row>
     <x:row r="55" ht="36" customHeight="1">
       <x:c r="A55" s="2" t="str">
-        <x:v>TU04</x:v>
+        <x:v>TU02</x:v>
       </x:c>
       <x:c r="B55" s="11" t="str">
-        <x:v>Produto repetido deve ser rejeitado antes do cálculo.</x:v>
+        <x:v>Sem cupom e sem fidelidade: total 5800 e zero pontos.</x:v>
       </x:c>
       <x:c r="C55" s="2" t="str">
         <x:v>APROVADO</x:v>
       </x:c>
       <x:c r="D55" s="8" t="n">
-        <x:v>0.058</x:v>
+        <x:v>0.159</x:v>
       </x:c>
       <x:c r="E55" s="2"/>
       <x:c r="F55" s="2"/>
@@ -3852,16 +3852,16 @@
     </x:row>
     <x:row r="56" ht="36" customHeight="1">
       <x:c r="A56" s="2" t="str">
-        <x:v>TU05</x:v>
+        <x:v>TU03</x:v>
       </x:c>
       <x:c r="B56" s="11" t="str">
-        <x:v>Rejeitar chave vazia, curta, excessiva ou com aspas.</x:v>
+        <x:v>Aceitar 1 e 10; rejeitar 0, -1, 11, 1.5, string e booleano.</x:v>
       </x:c>
       <x:c r="C56" s="2" t="str">
         <x:v>APROVADO</x:v>
       </x:c>
       <x:c r="D56" s="8" t="n">
-        <x:v>0.088</x:v>
+        <x:v>0.339</x:v>
       </x:c>
       <x:c r="E56" s="2"/>
       <x:c r="F56" s="2"/>
@@ -3870,16 +3870,16 @@
     </x:row>
     <x:row r="57" ht="36" customHeight="1">
       <x:c r="A57" s="2" t="str">
-        <x:v>TU06</x:v>
+        <x:v>TU04</x:v>
       </x:c>
       <x:c r="B57" s="11" t="str">
-        <x:v>Campos extras e corpo não estruturado são rejeitados.</x:v>
+        <x:v>Produto repetido deve ser rejeitado antes do cálculo.</x:v>
       </x:c>
       <x:c r="C57" s="2" t="str">
         <x:v>APROVADO</x:v>
       </x:c>
       <x:c r="D57" s="8" t="n">
-        <x:v>0.081</x:v>
+        <x:v>0.073</x:v>
       </x:c>
       <x:c r="E57" s="2"/>
       <x:c r="F57" s="2"/>
@@ -3888,16 +3888,16 @@
     </x:row>
     <x:row r="58" ht="36" customHeight="1">
       <x:c r="A58" s="2" t="str">
-        <x:v>UI01</x:v>
+        <x:v>TU05</x:v>
       </x:c>
       <x:c r="B58" s="11" t="str">
-        <x:v>Compra com desconto, fidelidade e confirmação preservada após falha do catálogo</x:v>
+        <x:v>Rejeitar chave vazia, curta, excessiva ou com aspas.</x:v>
       </x:c>
       <x:c r="C58" s="2" t="str">
         <x:v>APROVADO</x:v>
       </x:c>
       <x:c r="D58" s="8" t="n">
-        <x:v>1541</x:v>
+        <x:v>0.141</x:v>
       </x:c>
       <x:c r="E58" s="2"/>
       <x:c r="F58" s="2"/>
@@ -3906,16 +3906,16 @@
     </x:row>
     <x:row r="59" ht="36" customHeight="1">
       <x:c r="A59" s="2" t="str">
-        <x:v>UI02</x:v>
+        <x:v>TU06</x:v>
       </x:c>
       <x:c r="B59" s="11" t="str">
-        <x:v>Carrinho vazio e cupom inválido exibem mensagens</x:v>
+        <x:v>Campos extras e corpo não estruturado são rejeitados.</x:v>
       </x:c>
       <x:c r="C59" s="2" t="str">
         <x:v>APROVADO</x:v>
       </x:c>
       <x:c r="D59" s="8" t="n">
-        <x:v>197</x:v>
+        <x:v>0.194</x:v>
       </x:c>
       <x:c r="E59" s="2"/>
       <x:c r="F59" s="2"/>
@@ -3924,16 +3924,16 @@
     </x:row>
     <x:row r="60" ht="36" customHeight="1">
       <x:c r="A60" s="2" t="str">
-        <x:v>UI03</x:v>
+        <x:v>UI01</x:v>
       </x:c>
       <x:c r="B60" s="11" t="str">
-        <x:v>Recusa de pagamento exibida no fluxo</x:v>
+        <x:v>Compra com desconto, fidelidade e confirmação preservada após falha do catálogo</x:v>
       </x:c>
       <x:c r="C60" s="2" t="str">
         <x:v>APROVADO</x:v>
       </x:c>
       <x:c r="D60" s="8" t="n">
-        <x:v>429</x:v>
+        <x:v>1651</x:v>
       </x:c>
       <x:c r="E60" s="2"/>
       <x:c r="F60" s="2"/>
@@ -3942,16 +3942,16 @@
     </x:row>
     <x:row r="61" ht="36" customHeight="1">
       <x:c r="A61" s="2" t="str">
-        <x:v>UI04</x:v>
+        <x:v>UI02</x:v>
       </x:c>
       <x:c r="B61" s="11" t="str">
-        <x:v>Pagamento sem resposta apresenta pendência e opções de conferência simulada</x:v>
+        <x:v>Carrinho vazio e cupom inválido exibem mensagens</x:v>
       </x:c>
       <x:c r="C61" s="2" t="str">
         <x:v>APROVADO</x:v>
       </x:c>
       <x:c r="D61" s="8" t="n">
-        <x:v>440</x:v>
+        <x:v>206</x:v>
       </x:c>
       <x:c r="E61" s="2"/>
       <x:c r="F61" s="2"/>
@@ -3960,16 +3960,16 @@
     </x:row>
     <x:row r="62" ht="36" customHeight="1">
       <x:c r="A62" s="2" t="str">
-        <x:v>UI05</x:v>
+        <x:v>UI03</x:v>
       </x:c>
       <x:c r="B62" s="11" t="str">
-        <x:v>Larguras 360, 390 e 768 sem rolagem horizontal e controles de quantidade com 44 px</x:v>
+        <x:v>Recusa de pagamento exibida no fluxo</x:v>
       </x:c>
       <x:c r="C62" s="2" t="str">
         <x:v>APROVADO</x:v>
       </x:c>
       <x:c r="D62" s="8" t="n">
-        <x:v>513</x:v>
+        <x:v>533</x:v>
       </x:c>
       <x:c r="E62" s="2"/>
       <x:c r="F62" s="2"/>
@@ -3978,16 +3978,16 @@
     </x:row>
     <x:row r="63" ht="36" customHeight="1">
       <x:c r="A63" s="2" t="str">
-        <x:v>UI06</x:v>
+        <x:v>UI04</x:v>
       </x:c>
       <x:c r="B63" s="11" t="str">
-        <x:v>Aviso de privacidade visível e fidelidade opcional desmarcada</x:v>
+        <x:v>Pagamento sem resposta apresenta pendência e opções de conferência simulada</x:v>
       </x:c>
       <x:c r="C63" s="2" t="str">
         <x:v>APROVADO</x:v>
       </x:c>
       <x:c r="D63" s="8" t="n">
-        <x:v>384</x:v>
+        <x:v>601</x:v>
       </x:c>
       <x:c r="E63" s="2"/>
       <x:c r="F63" s="2"/>
@@ -3996,16 +3996,16 @@
     </x:row>
     <x:row r="64" ht="36" customHeight="1">
       <x:c r="A64" s="2" t="str">
-        <x:v>UI07</x:v>
+        <x:v>UI05</x:v>
       </x:c>
       <x:c r="B64" s="11" t="str">
-        <x:v>Controles ficam bloqueados durante o envio e até iniciar novo pedido</x:v>
+        <x:v>Larguras 360, 390 e 768 sem rolagem horizontal e controles de quantidade com 44 px</x:v>
       </x:c>
       <x:c r="C64" s="2" t="str">
         <x:v>APROVADO</x:v>
       </x:c>
       <x:c r="D64" s="8" t="n">
-        <x:v>203</x:v>
+        <x:v>771</x:v>
       </x:c>
       <x:c r="E64" s="2"/>
       <x:c r="F64" s="2"/>
@@ -4014,16 +4014,16 @@
     </x:row>
     <x:row r="65" ht="36" customHeight="1">
       <x:c r="A65" s="2" t="str">
-        <x:v>UI08</x:v>
+        <x:v>UI06</x:v>
       </x:c>
       <x:c r="B65" s="11" t="str">
-        <x:v>Resposta perdida permite repetir o mesmo pedido sem nova baixa de estoque</x:v>
+        <x:v>Aviso de privacidade visível e fidelidade opcional desmarcada</x:v>
       </x:c>
       <x:c r="C65" s="2" t="str">
         <x:v>APROVADO</x:v>
       </x:c>
       <x:c r="D65" s="8" t="n">
-        <x:v>213</x:v>
+        <x:v>596</x:v>
       </x:c>
       <x:c r="E65" s="2"/>
       <x:c r="F65" s="2"/>
@@ -4032,16 +4032,16 @@
     </x:row>
     <x:row r="66" ht="36" customHeight="1">
       <x:c r="A66" s="2" t="str">
-        <x:v>UI09</x:v>
+        <x:v>UI07</x:v>
       </x:c>
       <x:c r="B66" s="11" t="str">
-        <x:v>Rascunho mantém unidade, canal, produtos, cupom, fidelidade e pagamento ao recarregar</x:v>
+        <x:v>Controles ficam bloqueados durante o envio e até iniciar novo pedido</x:v>
       </x:c>
       <x:c r="C66" s="2" t="str">
         <x:v>APROVADO</x:v>
       </x:c>
       <x:c r="D66" s="8" t="n">
-        <x:v>252</x:v>
+        <x:v>271</x:v>
       </x:c>
       <x:c r="E66" s="2"/>
       <x:c r="F66" s="2"/>
@@ -4050,16 +4050,16 @@
     </x:row>
     <x:row r="67" ht="36" customHeight="1">
       <x:c r="A67" s="2" t="str">
-        <x:v>UI10</x:v>
+        <x:v>UI08</x:v>
       </x:c>
       <x:c r="B67" s="11" t="str">
-        <x:v>Confirmação reaparece ao recarregar e novo pedido libera os controles</x:v>
+        <x:v>Resposta perdida permite repetir o mesmo pedido sem nova baixa de estoque</x:v>
       </x:c>
       <x:c r="C67" s="2" t="str">
         <x:v>APROVADO</x:v>
       </x:c>
       <x:c r="D67" s="8" t="n">
-        <x:v>311</x:v>
+        <x:v>270</x:v>
       </x:c>
       <x:c r="E67" s="2"/>
       <x:c r="F67" s="2"/>
@@ -4068,16 +4068,16 @@
     </x:row>
     <x:row r="68" ht="36" customHeight="1">
       <x:c r="A68" s="2" t="str">
-        <x:v>UI11</x:v>
+        <x:v>UI09</x:v>
       </x:c>
       <x:c r="B68" s="11" t="str">
-        <x:v>Pendência sobrevive à recarga e pode ser aprovada ou recusada sem duplicar estoque e pontos</x:v>
+        <x:v>Rascunho mantém unidade, canal, produtos, cupom, fidelidade e pagamento ao recarregar</x:v>
       </x:c>
       <x:c r="C68" s="2" t="str">
         <x:v>APROVADO</x:v>
       </x:c>
       <x:c r="D68" s="8" t="n">
-        <x:v>629</x:v>
+        <x:v>374</x:v>
       </x:c>
       <x:c r="E68" s="2"/>
       <x:c r="F68" s="2"/>
@@ -4086,16 +4086,16 @@
     </x:row>
     <x:row r="69" ht="36" customHeight="1">
       <x:c r="A69" s="2" t="str">
-        <x:v>UI12</x:v>
+        <x:v>UI10</x:v>
       </x:c>
       <x:c r="B69" s="11" t="str">
-        <x:v>Resposta perdida e recarga preservam o corpo e a chave para recuperar a mesma compra</x:v>
+        <x:v>Confirmação reaparece ao recarregar e novo pedido libera os controles</x:v>
       </x:c>
       <x:c r="C69" s="2" t="str">
         <x:v>APROVADO</x:v>
       </x:c>
       <x:c r="D69" s="8" t="n">
-        <x:v>250</x:v>
+        <x:v>457</x:v>
       </x:c>
       <x:c r="E69" s="2"/>
       <x:c r="F69" s="2"/>
@@ -4104,16 +4104,16 @@
     </x:row>
     <x:row r="70" ht="36" customHeight="1">
       <x:c r="A70" s="2" t="str">
-        <x:v>UI13</x:v>
+        <x:v>UI11</x:v>
       </x:c>
       <x:c r="B70" s="11" t="str">
-        <x:v>Falhas de catálogo impedem compra com dados antigos e permitem nova tentativa</x:v>
+        <x:v>Pendência sobrevive à recarga e pode ser aprovada ou recusada sem duplicar estoque e pontos</x:v>
       </x:c>
       <x:c r="C70" s="2" t="str">
         <x:v>APROVADO</x:v>
       </x:c>
       <x:c r="D70" s="8" t="n">
-        <x:v>1949</x:v>
+        <x:v>905</x:v>
       </x:c>
       <x:c r="E70" s="2"/>
       <x:c r="F70" s="2"/>
@@ -4122,16 +4122,16 @@
     </x:row>
     <x:row r="71" ht="36" customHeight="1">
       <x:c r="A71" s="2" t="str">
-        <x:v>UI14</x:v>
+        <x:v>UI12</x:v>
       </x:c>
       <x:c r="B71" s="11" t="str">
-        <x:v>Quantidade respeita estoque e limite de dez, com botões desabilitados nos limites</x:v>
+        <x:v>Resposta perdida e recarga preservam o corpo e a chave para recuperar a mesma compra</x:v>
       </x:c>
       <x:c r="C71" s="2" t="str">
         <x:v>APROVADO</x:v>
       </x:c>
       <x:c r="D71" s="8" t="n">
-        <x:v>409</x:v>
+        <x:v>328</x:v>
       </x:c>
       <x:c r="E71" s="2"/>
       <x:c r="F71" s="2"/>
@@ -4140,16 +4140,16 @@
     </x:row>
     <x:row r="72" ht="36" customHeight="1">
       <x:c r="A72" s="2" t="str">
-        <x:v>UI15</x:v>
+        <x:v>UI13</x:v>
       </x:c>
       <x:c r="B72" s="11" t="str">
-        <x:v>Envio sem resposta termina em oito segundos e repete a compra sem duplicação</x:v>
+        <x:v>Falhas de catálogo impedem compra com dados antigos e permitem nova tentativa</x:v>
       </x:c>
       <x:c r="C72" s="2" t="str">
         <x:v>APROVADO</x:v>
       </x:c>
       <x:c r="D72" s="8" t="n">
-        <x:v>8679</x:v>
+        <x:v>2029</x:v>
       </x:c>
       <x:c r="E72" s="2"/>
       <x:c r="F72" s="2"/>
@@ -4158,16 +4158,16 @@
     </x:row>
     <x:row r="73" ht="36" customHeight="1">
       <x:c r="A73" s="2" t="str">
-        <x:v>UI16</x:v>
+        <x:v>UI14</x:v>
       </x:c>
       <x:c r="B73" s="11" t="str">
-        <x:v>Sessão expirada pode ser atualizada preservando a tentativa de compra</x:v>
+        <x:v>Quantidade respeita estoque e limite de dez, com botões desabilitados nos limites</x:v>
       </x:c>
       <x:c r="C73" s="2" t="str">
         <x:v>APROVADO</x:v>
       </x:c>
       <x:c r="D73" s="8" t="n">
-        <x:v>259</x:v>
+        <x:v>613</x:v>
       </x:c>
       <x:c r="E73" s="2"/>
       <x:c r="F73" s="2"/>
@@ -4176,16 +4176,16 @@
     </x:row>
     <x:row r="74" ht="36" customHeight="1">
       <x:c r="A74" s="2" t="str">
-        <x:v>UI17</x:v>
+        <x:v>UI15</x:v>
       </x:c>
       <x:c r="B74" s="11" t="str">
-        <x:v>Recarregar durante o envio recupera o mesmo pedido sem uma nova compra</x:v>
+        <x:v>Envio sem resposta termina em oito segundos e repete a compra sem duplicação</x:v>
       </x:c>
       <x:c r="C74" s="2" t="str">
         <x:v>APROVADO</x:v>
       </x:c>
       <x:c r="D74" s="8" t="n">
-        <x:v>268</x:v>
+        <x:v>8725</x:v>
       </x:c>
       <x:c r="E74" s="2"/>
       <x:c r="F74" s="2"/>
@@ -4194,37 +4194,53 @@
     </x:row>
     <x:row r="75" ht="36" customHeight="1">
       <x:c r="A75" s="2" t="str">
-        <x:v>UI18</x:v>
+        <x:v>UI16</x:v>
       </x:c>
       <x:c r="B75" s="11" t="str">
-        <x:v>Resposta perdida na conferência bloqueia a opção oposta e recarga recupera a aprovação</x:v>
+        <x:v>Sessão expirada pode ser atualizada preservando a tentativa de compra</x:v>
       </x:c>
       <x:c r="C75" s="2" t="str">
         <x:v>APROVADO</x:v>
       </x:c>
       <x:c r="D75" s="8" t="n">
-        <x:v>324</x:v>
+        <x:v>275</x:v>
       </x:c>
       <x:c r="E75" s="2"/>
       <x:c r="F75" s="2"/>
       <x:c r="G75" s="2"/>
       <x:c r="H75" s="2"/>
     </x:row>
-    <x:row r="76">
-      <x:c r="A76" s="2"/>
-      <x:c r="B76" s="2"/>
-      <x:c r="C76" s="2"/>
-      <x:c r="D76" s="2"/>
+    <x:row r="76" ht="36" customHeight="1">
+      <x:c r="A76" s="2" t="str">
+        <x:v>UI17</x:v>
+      </x:c>
+      <x:c r="B76" s="11" t="str">
+        <x:v>Recarregar durante o envio recupera o mesmo pedido sem uma nova compra</x:v>
+      </x:c>
+      <x:c r="C76" s="2" t="str">
+        <x:v>APROVADO</x:v>
+      </x:c>
+      <x:c r="D76" s="8" t="n">
+        <x:v>251</x:v>
+      </x:c>
       <x:c r="E76" s="2"/>
       <x:c r="F76" s="2"/>
       <x:c r="G76" s="2"/>
       <x:c r="H76" s="2"/>
     </x:row>
-    <x:row r="77">
-      <x:c r="A77" s="2"/>
-      <x:c r="B77" s="2"/>
-      <x:c r="C77" s="2"/>
-      <x:c r="D77" s="2"/>
+    <x:row r="77" ht="36" customHeight="1">
+      <x:c r="A77" s="2" t="str">
+        <x:v>UI18</x:v>
+      </x:c>
+      <x:c r="B77" s="11" t="str">
+        <x:v>Resposta perdida na conferência bloqueia a opção oposta e recarga recupera a aprovação</x:v>
+      </x:c>
+      <x:c r="C77" s="2" t="str">
+        <x:v>APROVADO</x:v>
+      </x:c>
+      <x:c r="D77" s="8" t="n">
+        <x:v>340</x:v>
+      </x:c>
       <x:c r="E77" s="2"/>
       <x:c r="F77" s="2"/>
       <x:c r="G77" s="2"/>
@@ -5841,7 +5857,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="B6" s="8" t="n">
-        <x:v>9.891</x:v>
+        <x:v>15.179</x:v>
       </x:c>
       <x:c r="C6" s="2" t="n">
         <x:v>1</x:v>
@@ -5857,7 +5873,7 @@
         <x:v>1</x:v>
       </x:c>
       <x:c r="B7" s="8" t="n">
-        <x:v>1204.152</x:v>
+        <x:v>775.284</x:v>
       </x:c>
       <x:c r="C7" s="2" t="n">
         <x:v>1</x:v>
@@ -5873,7 +5889,7 @@
         <x:v>2</x:v>
       </x:c>
       <x:c r="B8" s="8" t="n">
-        <x:v>56.848</x:v>
+        <x:v>17.436</x:v>
       </x:c>
       <x:c r="C8" s="2" t="n">
         <x:v>1</x:v>
@@ -5889,7 +5905,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="B9" s="8" t="n">
-        <x:v>768.637</x:v>
+        <x:v>32.845</x:v>
       </x:c>
       <x:c r="C9" s="2" t="n">
         <x:v>1</x:v>
@@ -5905,7 +5921,7 @@
         <x:v>4</x:v>
       </x:c>
       <x:c r="B10" s="8" t="n">
-        <x:v>25.321</x:v>
+        <x:v>141.07</x:v>
       </x:c>
       <x:c r="C10" s="2" t="n">
         <x:v>1</x:v>
@@ -5921,7 +5937,7 @@
         <x:v>5</x:v>
       </x:c>
       <x:c r="B11" s="8" t="n">
-        <x:v>12.714</x:v>
+        <x:v>23.719</x:v>
       </x:c>
       <x:c r="C11" s="2" t="n">
         <x:v>1</x:v>
@@ -5937,7 +5953,7 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="B12" s="8" t="n">
-        <x:v>25.473</x:v>
+        <x:v>60.781</x:v>
       </x:c>
       <x:c r="C12" s="2" t="n">
         <x:v>1</x:v>
@@ -5953,7 +5969,7 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="B13" s="8" t="n">
-        <x:v>162.606</x:v>
+        <x:v>123.169</x:v>
       </x:c>
       <x:c r="C13" s="2" t="n">
         <x:v>1</x:v>
@@ -5969,7 +5985,7 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="B14" s="8" t="n">
-        <x:v>84.118</x:v>
+        <x:v>75.35</x:v>
       </x:c>
       <x:c r="C14" s="2" t="n">
         <x:v>1</x:v>
@@ -5985,7 +6001,7 @@
         <x:v>9</x:v>
       </x:c>
       <x:c r="B15" s="8" t="n">
-        <x:v>37.529</x:v>
+        <x:v>23.612</x:v>
       </x:c>
       <x:c r="C15" s="2" t="n">
         <x:v>1</x:v>
@@ -6001,7 +6017,7 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="B16" s="8" t="n">
-        <x:v>63.218</x:v>
+        <x:v>22.472</x:v>
       </x:c>
       <x:c r="C16" s="2" t="n">
         <x:v>1</x:v>
@@ -6017,7 +6033,7 @@
         <x:v>11</x:v>
       </x:c>
       <x:c r="B17" s="8" t="n">
-        <x:v>19.297</x:v>
+        <x:v>78.62</x:v>
       </x:c>
       <x:c r="C17" s="2" t="n">
         <x:v>1</x:v>
@@ -6033,7 +6049,7 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="B18" s="8" t="n">
-        <x:v>19.402</x:v>
+        <x:v>286.47</x:v>
       </x:c>
       <x:c r="C18" s="2" t="n">
         <x:v>1</x:v>
@@ -6049,7 +6065,7 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="B19" s="8" t="n">
-        <x:v>10.549</x:v>
+        <x:v>10.172</x:v>
       </x:c>
       <x:c r="C19" s="2" t="n">
         <x:v>1</x:v>
@@ -6065,7 +6081,7 @@
         <x:v>14</x:v>
       </x:c>
       <x:c r="B20" s="8" t="n">
-        <x:v>147.364</x:v>
+        <x:v>14.848</x:v>
       </x:c>
       <x:c r="C20" s="2" t="n">
         <x:v>1</x:v>
@@ -6081,7 +6097,7 @@
         <x:v>15</x:v>
       </x:c>
       <x:c r="B21" s="8" t="n">
-        <x:v>21.131</x:v>
+        <x:v>73.883</x:v>
       </x:c>
       <x:c r="C21" s="2" t="n">
         <x:v>1</x:v>
@@ -6097,7 +6113,7 @@
         <x:v>16</x:v>
       </x:c>
       <x:c r="B22" s="8" t="n">
-        <x:v>11.001</x:v>
+        <x:v>17.799</x:v>
       </x:c>
       <x:c r="C22" s="2" t="n">
         <x:v>1</x:v>
@@ -6113,7 +6129,7 @@
         <x:v>17</x:v>
       </x:c>
       <x:c r="B23" s="8" t="n">
-        <x:v>34.122</x:v>
+        <x:v>34.088</x:v>
       </x:c>
       <x:c r="C23" s="2" t="n">
         <x:v>1</x:v>
@@ -6129,7 +6145,7 @@
         <x:v>18</x:v>
       </x:c>
       <x:c r="B24" s="8" t="n">
-        <x:v>14.721</x:v>
+        <x:v>16.336</x:v>
       </x:c>
       <x:c r="C24" s="2" t="n">
         <x:v>1</x:v>
@@ -6145,7 +6161,7 @@
         <x:v>19</x:v>
       </x:c>
       <x:c r="B25" s="8" t="n">
-        <x:v>77.218</x:v>
+        <x:v>58.985</x:v>
       </x:c>
       <x:c r="C25" s="2" t="n">
         <x:v>1</x:v>
@@ -6161,7 +6177,7 @@
         <x:v>20</x:v>
       </x:c>
       <x:c r="B26" s="8" t="n">
-        <x:v>59.67</x:v>
+        <x:v>19.11</x:v>
       </x:c>
       <x:c r="C26" s="2" t="n">
         <x:v>1</x:v>
@@ -6177,7 +6193,7 @@
         <x:v>21</x:v>
       </x:c>
       <x:c r="B27" s="8" t="n">
-        <x:v>82.773</x:v>
+        <x:v>23.502</x:v>
       </x:c>
       <x:c r="C27" s="2" t="n">
         <x:v>1</x:v>
@@ -6193,7 +6209,7 @@
         <x:v>22</x:v>
       </x:c>
       <x:c r="B28" s="8" t="n">
-        <x:v>29.67</x:v>
+        <x:v>322.435</x:v>
       </x:c>
       <x:c r="C28" s="2" t="n">
         <x:v>1</x:v>
@@ -6209,7 +6225,7 @@
         <x:v>23</x:v>
       </x:c>
       <x:c r="B29" s="8" t="n">
-        <x:v>547.64</x:v>
+        <x:v>94.875</x:v>
       </x:c>
       <x:c r="C29" s="2" t="n">
         <x:v>1</x:v>
@@ -6225,7 +6241,7 @@
         <x:v>24</x:v>
       </x:c>
       <x:c r="B30" s="8" t="n">
-        <x:v>6.369</x:v>
+        <x:v>18.186</x:v>
       </x:c>
       <x:c r="C30" s="2" t="n">
         <x:v>1</x:v>
@@ -6241,7 +6257,7 @@
         <x:v>25</x:v>
       </x:c>
       <x:c r="B31" s="8" t="n">
-        <x:v>11.682</x:v>
+        <x:v>61.471</x:v>
       </x:c>
       <x:c r="C31" s="2" t="n">
         <x:v>1</x:v>
@@ -6257,7 +6273,7 @@
         <x:v>26</x:v>
       </x:c>
       <x:c r="B32" s="8" t="n">
-        <x:v>28.122</x:v>
+        <x:v>27.79</x:v>
       </x:c>
       <x:c r="C32" s="2" t="n">
         <x:v>1</x:v>
@@ -6273,7 +6289,7 @@
         <x:v>27</x:v>
       </x:c>
       <x:c r="B33" s="8" t="n">
-        <x:v>9.486</x:v>
+        <x:v>18.46</x:v>
       </x:c>
       <x:c r="C33" s="2" t="n">
         <x:v>1</x:v>
@@ -6289,7 +6305,7 @@
         <x:v>28</x:v>
       </x:c>
       <x:c r="B34" s="8" t="n">
-        <x:v>11.092</x:v>
+        <x:v>59.859</x:v>
       </x:c>
       <x:c r="C34" s="2" t="n">
         <x:v>1</x:v>
@@ -6305,7 +6321,7 @@
         <x:v>29</x:v>
       </x:c>
       <x:c r="B35" s="8" t="n">
-        <x:v>18.565</x:v>
+        <x:v>46.629</x:v>
       </x:c>
       <x:c r="C35" s="2" t="n">
         <x:v>1</x:v>
@@ -6321,7 +6337,7 @@
         <x:v>30</x:v>
       </x:c>
       <x:c r="B36" s="8" t="n">
-        <x:v>18.212</x:v>
+        <x:v>13.592</x:v>
       </x:c>
       <x:c r="C36" s="2" t="n">
         <x:v>1</x:v>
@@ -6337,7 +6353,7 @@
         <x:v>31</x:v>
       </x:c>
       <x:c r="B37" s="8" t="n">
-        <x:v>37.72</x:v>
+        <x:v>17.217</x:v>
       </x:c>
       <x:c r="C37" s="2" t="n">
         <x:v>1</x:v>
@@ -6353,7 +6369,7 @@
         <x:v>32</x:v>
       </x:c>
       <x:c r="B38" s="8" t="n">
-        <x:v>18.541</x:v>
+        <x:v>91.059</x:v>
       </x:c>
       <x:c r="C38" s="2" t="n">
         <x:v>1</x:v>
@@ -6369,7 +6385,7 @@
         <x:v>33</x:v>
       </x:c>
       <x:c r="B39" s="8" t="n">
-        <x:v>49.09</x:v>
+        <x:v>1108.249</x:v>
       </x:c>
       <x:c r="C39" s="2" t="n">
         <x:v>1</x:v>
@@ -6385,7 +6401,7 @@
         <x:v>34</x:v>
       </x:c>
       <x:c r="B40" s="8" t="n">
-        <x:v>16.392</x:v>
+        <x:v>93.675</x:v>
       </x:c>
       <x:c r="C40" s="2" t="n">
         <x:v>1</x:v>
@@ -6401,7 +6417,7 @@
         <x:v>35</x:v>
       </x:c>
       <x:c r="B41" s="8" t="n">
-        <x:v>43.66</x:v>
+        <x:v>37.686</x:v>
       </x:c>
       <x:c r="C41" s="2" t="n">
         <x:v>1</x:v>
@@ -6417,7 +6433,7 @@
         <x:v>36</x:v>
       </x:c>
       <x:c r="B42" s="8" t="n">
-        <x:v>22.028</x:v>
+        <x:v>91.101</x:v>
       </x:c>
       <x:c r="C42" s="2" t="n">
         <x:v>1</x:v>
@@ -6433,7 +6449,7 @@
         <x:v>37</x:v>
       </x:c>
       <x:c r="B43" s="8" t="n">
-        <x:v>49.873</x:v>
+        <x:v>14.491</x:v>
       </x:c>
       <x:c r="C43" s="2" t="n">
         <x:v>1</x:v>
@@ -6449,7 +6465,7 @@
         <x:v>38</x:v>
       </x:c>
       <x:c r="B44" s="8" t="n">
-        <x:v>30.748</x:v>
+        <x:v>30.65</x:v>
       </x:c>
       <x:c r="C44" s="2" t="n">
         <x:v>1</x:v>
@@ -6465,7 +6481,7 @@
         <x:v>39</x:v>
       </x:c>
       <x:c r="B45" s="8" t="n">
-        <x:v>31.41</x:v>
+        <x:v>11.51</x:v>
       </x:c>
       <x:c r="C45" s="2" t="n">
         <x:v>1</x:v>
@@ -6481,7 +6497,7 @@
         <x:v>40</x:v>
       </x:c>
       <x:c r="B46" s="8" t="n">
-        <x:v>52.363</x:v>
+        <x:v>94.424</x:v>
       </x:c>
       <x:c r="C46" s="2" t="n">
         <x:v>1</x:v>
@@ -6497,7 +6513,7 @@
         <x:v>41</x:v>
       </x:c>
       <x:c r="B47" s="8" t="n">
-        <x:v>77.151</x:v>
+        <x:v>18.577</x:v>
       </x:c>
       <x:c r="C47" s="2" t="n">
         <x:v>1</x:v>
@@ -6513,7 +6529,7 @@
         <x:v>42</x:v>
       </x:c>
       <x:c r="B48" s="8" t="n">
-        <x:v>28.917</x:v>
+        <x:v>17.279</x:v>
       </x:c>
       <x:c r="C48" s="2" t="n">
         <x:v>1</x:v>
@@ -6529,7 +6545,7 @@
         <x:v>43</x:v>
       </x:c>
       <x:c r="B49" s="8" t="n">
-        <x:v>294.83</x:v>
+        <x:v>16.489</x:v>
       </x:c>
       <x:c r="C49" s="2" t="n">
         <x:v>1</x:v>
@@ -6545,7 +6561,7 @@
         <x:v>44</x:v>
       </x:c>
       <x:c r="B50" s="8" t="n">
-        <x:v>11.653</x:v>
+        <x:v>18.593</x:v>
       </x:c>
       <x:c r="C50" s="2" t="n">
         <x:v>1</x:v>
@@ -6561,7 +6577,7 @@
         <x:v>45</x:v>
       </x:c>
       <x:c r="B51" s="8" t="n">
-        <x:v>22.102</x:v>
+        <x:v>23.506</x:v>
       </x:c>
       <x:c r="C51" s="2" t="n">
         <x:v>1</x:v>
@@ -6577,7 +6593,7 @@
         <x:v>46</x:v>
       </x:c>
       <x:c r="B52" s="8" t="n">
-        <x:v>34.949</x:v>
+        <x:v>23.044</x:v>
       </x:c>
       <x:c r="C52" s="2" t="n">
         <x:v>1</x:v>
@@ -6593,7 +6609,7 @@
         <x:v>47</x:v>
       </x:c>
       <x:c r="B53" s="8" t="n">
-        <x:v>340.544</x:v>
+        <x:v>24.445</x:v>
       </x:c>
       <x:c r="C53" s="2" t="n">
         <x:v>1</x:v>
@@ -6609,7 +6625,7 @@
         <x:v>48</x:v>
       </x:c>
       <x:c r="B54" s="8" t="n">
-        <x:v>89.044</x:v>
+        <x:v>42.758</x:v>
       </x:c>
       <x:c r="C54" s="2" t="n">
         <x:v>1</x:v>
@@ -6625,7 +6641,7 @@
         <x:v>49</x:v>
       </x:c>
       <x:c r="B55" s="8" t="n">
-        <x:v>13.638</x:v>
+        <x:v>27.362</x:v>
       </x:c>
       <x:c r="C55" s="2" t="n">
         <x:v>1</x:v>
@@ -6641,7 +6657,7 @@
         <x:v>50</x:v>
       </x:c>
       <x:c r="B56" s="8" t="n">
-        <x:v>45.328</x:v>
+        <x:v>36.66</x:v>
       </x:c>
       <x:c r="C56" s="2" t="n">
         <x:v>1</x:v>
@@ -6657,7 +6673,7 @@
         <x:v>51</x:v>
       </x:c>
       <x:c r="B57" s="8" t="n">
-        <x:v>9.667</x:v>
+        <x:v>12.11</x:v>
       </x:c>
       <x:c r="C57" s="2" t="n">
         <x:v>1</x:v>
@@ -6673,7 +6689,7 @@
         <x:v>52</x:v>
       </x:c>
       <x:c r="B58" s="8" t="n">
-        <x:v>13.01</x:v>
+        <x:v>51.04</x:v>
       </x:c>
       <x:c r="C58" s="2" t="n">
         <x:v>1</x:v>
@@ -6689,7 +6705,7 @@
         <x:v>53</x:v>
       </x:c>
       <x:c r="B59" s="8" t="n">
-        <x:v>43.096</x:v>
+        <x:v>62.425</x:v>
       </x:c>
       <x:c r="C59" s="2" t="n">
         <x:v>1</x:v>
@@ -6705,7 +6721,7 @@
         <x:v>54</x:v>
       </x:c>
       <x:c r="B60" s="8" t="n">
-        <x:v>10.495</x:v>
+        <x:v>22.172</x:v>
       </x:c>
       <x:c r="C60" s="2" t="n">
         <x:v>1</x:v>
@@ -6721,7 +6737,7 @@
         <x:v>55</x:v>
       </x:c>
       <x:c r="B61" s="8" t="n">
-        <x:v>107.598</x:v>
+        <x:v>32.982</x:v>
       </x:c>
       <x:c r="C61" s="2" t="n">
         <x:v>1</x:v>
@@ -6737,7 +6753,7 @@
         <x:v>56</x:v>
       </x:c>
       <x:c r="B62" s="8" t="n">
-        <x:v>29.378</x:v>
+        <x:v>34.135</x:v>
       </x:c>
       <x:c r="C62" s="2" t="n">
         <x:v>1</x:v>
@@ -6753,7 +6769,7 @@
         <x:v>57</x:v>
       </x:c>
       <x:c r="B63" s="8" t="n">
-        <x:v>9.4</x:v>
+        <x:v>14.48</x:v>
       </x:c>
       <x:c r="C63" s="2" t="n">
         <x:v>1</x:v>
@@ -6769,7 +6785,7 @@
         <x:v>58</x:v>
       </x:c>
       <x:c r="B64" s="8" t="n">
-        <x:v>29.769</x:v>
+        <x:v>38.336</x:v>
       </x:c>
       <x:c r="C64" s="2" t="n">
         <x:v>1</x:v>
@@ -6785,7 +6801,7 @@
         <x:v>59</x:v>
       </x:c>
       <x:c r="B65" s="8" t="n">
-        <x:v>61.878</x:v>
+        <x:v>40.528</x:v>
       </x:c>
       <x:c r="C65" s="2" t="n">
         <x:v>1</x:v>
@@ -6801,7 +6817,7 @@
         <x:v>60</x:v>
       </x:c>
       <x:c r="B66" s="8" t="n">
-        <x:v>24.202</x:v>
+        <x:v>43.332</x:v>
       </x:c>
       <x:c r="C66" s="2" t="n">
         <x:v>1</x:v>
@@ -6817,7 +6833,7 @@
         <x:v>61</x:v>
       </x:c>
       <x:c r="B67" s="8" t="n">
-        <x:v>22.874</x:v>
+        <x:v>13.455</x:v>
       </x:c>
       <x:c r="C67" s="2" t="n">
         <x:v>1</x:v>
@@ -6833,7 +6849,7 @@
         <x:v>62</x:v>
       </x:c>
       <x:c r="B68" s="8" t="n">
-        <x:v>11.282</x:v>
+        <x:v>38.977</x:v>
       </x:c>
       <x:c r="C68" s="2" t="n">
         <x:v>1</x:v>
@@ -6849,7 +6865,7 @@
         <x:v>63</x:v>
       </x:c>
       <x:c r="B69" s="8" t="n">
-        <x:v>14.006</x:v>
+        <x:v>48.456</x:v>
       </x:c>
       <x:c r="C69" s="2" t="n">
         <x:v>1</x:v>
@@ -6865,7 +6881,7 @@
         <x:v>64</x:v>
       </x:c>
       <x:c r="B70" s="8" t="n">
-        <x:v>58.364</x:v>
+        <x:v>33.826</x:v>
       </x:c>
       <x:c r="C70" s="2" t="n">
         <x:v>1</x:v>
@@ -6881,7 +6897,7 @@
         <x:v>65</x:v>
       </x:c>
       <x:c r="B71" s="8" t="n">
-        <x:v>12.307</x:v>
+        <x:v>47.384</x:v>
       </x:c>
       <x:c r="C71" s="2" t="n">
         <x:v>1</x:v>
@@ -6897,7 +6913,7 @@
         <x:v>66</x:v>
       </x:c>
       <x:c r="B72" s="8" t="n">
-        <x:v>11.947</x:v>
+        <x:v>47.091</x:v>
       </x:c>
       <x:c r="C72" s="2" t="n">
         <x:v>1</x:v>
@@ -6913,7 +6929,7 @@
         <x:v>67</x:v>
       </x:c>
       <x:c r="B73" s="8" t="n">
-        <x:v>13.407</x:v>
+        <x:v>21.565</x:v>
       </x:c>
       <x:c r="C73" s="2" t="n">
         <x:v>1</x:v>
@@ -6929,7 +6945,7 @@
         <x:v>68</x:v>
       </x:c>
       <x:c r="B74" s="8" t="n">
-        <x:v>42.274</x:v>
+        <x:v>27.875</x:v>
       </x:c>
       <x:c r="C74" s="2" t="n">
         <x:v>1</x:v>
@@ -6945,7 +6961,7 @@
         <x:v>69</x:v>
       </x:c>
       <x:c r="B75" s="8" t="n">
-        <x:v>9.505</x:v>
+        <x:v>35.802</x:v>
       </x:c>
       <x:c r="C75" s="2" t="n">
         <x:v>1</x:v>
@@ -6961,7 +6977,7 @@
         <x:v>70</x:v>
       </x:c>
       <x:c r="B76" s="8" t="n">
-        <x:v>42.745</x:v>
+        <x:v>36.456</x:v>
       </x:c>
       <x:c r="C76" s="2" t="n">
         <x:v>1</x:v>
@@ -6977,7 +6993,7 @@
         <x:v>71</x:v>
       </x:c>
       <x:c r="B77" s="8" t="n">
-        <x:v>13.829</x:v>
+        <x:v>75.362</x:v>
       </x:c>
       <x:c r="C77" s="2" t="n">
         <x:v>1</x:v>
@@ -6993,7 +7009,7 @@
         <x:v>72</x:v>
       </x:c>
       <x:c r="B78" s="8" t="n">
-        <x:v>60.094</x:v>
+        <x:v>84.035</x:v>
       </x:c>
       <x:c r="C78" s="2" t="n">
         <x:v>1</x:v>
@@ -7009,7 +7025,7 @@
         <x:v>73</x:v>
       </x:c>
       <x:c r="B79" s="8" t="n">
-        <x:v>208.004</x:v>
+        <x:v>30.757</x:v>
       </x:c>
       <x:c r="C79" s="2" t="n">
         <x:v>1</x:v>
@@ -7025,7 +7041,7 @@
         <x:v>74</x:v>
       </x:c>
       <x:c r="B80" s="8" t="n">
-        <x:v>59.835</x:v>
+        <x:v>38.145</x:v>
       </x:c>
       <x:c r="C80" s="2" t="n">
         <x:v>1</x:v>
@@ -7041,7 +7057,7 @@
         <x:v>75</x:v>
       </x:c>
       <x:c r="B81" s="8" t="n">
-        <x:v>11.86</x:v>
+        <x:v>39.755</x:v>
       </x:c>
       <x:c r="C81" s="2" t="n">
         <x:v>1</x:v>
@@ -7057,7 +7073,7 @@
         <x:v>76</x:v>
       </x:c>
       <x:c r="B82" s="8" t="n">
-        <x:v>14.196</x:v>
+        <x:v>40.017</x:v>
       </x:c>
       <x:c r="C82" s="2" t="n">
         <x:v>1</x:v>
@@ -7073,7 +7089,7 @@
         <x:v>77</x:v>
       </x:c>
       <x:c r="B83" s="8" t="n">
-        <x:v>17.122</x:v>
+        <x:v>55.774</x:v>
       </x:c>
       <x:c r="C83" s="2" t="n">
         <x:v>1</x:v>
@@ -7089,7 +7105,7 @@
         <x:v>78</x:v>
       </x:c>
       <x:c r="B84" s="8" t="n">
-        <x:v>47.508</x:v>
+        <x:v>43.094</x:v>
       </x:c>
       <x:c r="C84" s="2" t="n">
         <x:v>1</x:v>
@@ -7105,7 +7121,7 @@
         <x:v>79</x:v>
       </x:c>
       <x:c r="B85" s="8" t="n">
-        <x:v>16.274</x:v>
+        <x:v>50.345</x:v>
       </x:c>
       <x:c r="C85" s="2" t="n">
         <x:v>1</x:v>
@@ -7121,7 +7137,7 @@
         <x:v>80</x:v>
       </x:c>
       <x:c r="B86" s="8" t="n">
-        <x:v>47.062</x:v>
+        <x:v>52.752</x:v>
       </x:c>
       <x:c r="C86" s="2" t="n">
         <x:v>1</x:v>
@@ -7137,7 +7153,7 @@
         <x:v>81</x:v>
       </x:c>
       <x:c r="B87" s="8" t="n">
-        <x:v>33.821</x:v>
+        <x:v>60.647</x:v>
       </x:c>
       <x:c r="C87" s="2" t="n">
         <x:v>1</x:v>
@@ -7153,7 +7169,7 @@
         <x:v>82</x:v>
       </x:c>
       <x:c r="B88" s="8" t="n">
-        <x:v>11.045</x:v>
+        <x:v>877.268</x:v>
       </x:c>
       <x:c r="C88" s="2" t="n">
         <x:v>1</x:v>
@@ -7169,7 +7185,7 @@
         <x:v>83</x:v>
       </x:c>
       <x:c r="B89" s="8" t="n">
-        <x:v>9.513</x:v>
+        <x:v>25.184</x:v>
       </x:c>
       <x:c r="C89" s="2" t="n">
         <x:v>1</x:v>
@@ -7185,7 +7201,7 @@
         <x:v>84</x:v>
       </x:c>
       <x:c r="B90" s="8" t="n">
-        <x:v>18.847</x:v>
+        <x:v>58.014</x:v>
       </x:c>
       <x:c r="C90" s="2" t="n">
         <x:v>1</x:v>
@@ -7201,7 +7217,7 @@
         <x:v>85</x:v>
       </x:c>
       <x:c r="B91" s="8" t="n">
-        <x:v>34.401</x:v>
+        <x:v>41.041</x:v>
       </x:c>
       <x:c r="C91" s="2" t="n">
         <x:v>1</x:v>
@@ -7217,7 +7233,7 @@
         <x:v>86</x:v>
       </x:c>
       <x:c r="B92" s="8" t="n">
-        <x:v>56.309</x:v>
+        <x:v>42.88</x:v>
       </x:c>
       <x:c r="C92" s="2" t="n">
         <x:v>1</x:v>
@@ -7233,7 +7249,7 @@
         <x:v>87</x:v>
       </x:c>
       <x:c r="B93" s="8" t="n">
-        <x:v>12.266</x:v>
+        <x:v>43.637</x:v>
       </x:c>
       <x:c r="C93" s="2" t="n">
         <x:v>1</x:v>
@@ -7249,7 +7265,7 @@
         <x:v>88</x:v>
       </x:c>
       <x:c r="B94" s="8" t="n">
-        <x:v>13.5</x:v>
+        <x:v>14.2</x:v>
       </x:c>
       <x:c r="C94" s="2" t="n">
         <x:v>1</x:v>
@@ -7265,7 +7281,7 @@
         <x:v>89</x:v>
       </x:c>
       <x:c r="B95" s="8" t="n">
-        <x:v>25.874</x:v>
+        <x:v>46.8</x:v>
       </x:c>
       <x:c r="C95" s="2" t="n">
         <x:v>1</x:v>
@@ -7281,7 +7297,7 @@
         <x:v>90</x:v>
       </x:c>
       <x:c r="B96" s="8" t="n">
-        <x:v>15.79</x:v>
+        <x:v>29.04</x:v>
       </x:c>
       <x:c r="C96" s="2" t="n">
         <x:v>1</x:v>
@@ -7297,7 +7313,7 @@
         <x:v>91</x:v>
       </x:c>
       <x:c r="B97" s="8" t="n">
-        <x:v>28.063</x:v>
+        <x:v>28.3</x:v>
       </x:c>
       <x:c r="C97" s="2" t="n">
         <x:v>1</x:v>
@@ -7313,7 +7329,7 @@
         <x:v>92</x:v>
       </x:c>
       <x:c r="B98" s="8" t="n">
-        <x:v>33.77</x:v>
+        <x:v>30.543</x:v>
       </x:c>
       <x:c r="C98" s="2" t="n">
         <x:v>1</x:v>
@@ -7329,7 +7345,7 @@
         <x:v>93</x:v>
       </x:c>
       <x:c r="B99" s="8" t="n">
-        <x:v>32.328</x:v>
+        <x:v>32.305</x:v>
       </x:c>
       <x:c r="C99" s="2" t="n">
         <x:v>1</x:v>
@@ -7345,7 +7361,7 @@
         <x:v>94</x:v>
       </x:c>
       <x:c r="B100" s="8" t="n">
-        <x:v>37.348</x:v>
+        <x:v>63.91</x:v>
       </x:c>
       <x:c r="C100" s="2" t="n">
         <x:v>1</x:v>
@@ -7361,7 +7377,7 @@
         <x:v>95</x:v>
       </x:c>
       <x:c r="B101" s="8" t="n">
-        <x:v>24.393</x:v>
+        <x:v>35.545</x:v>
       </x:c>
       <x:c r="C101" s="2" t="n">
         <x:v>1</x:v>
@@ -7377,7 +7393,7 @@
         <x:v>96</x:v>
       </x:c>
       <x:c r="B102" s="8" t="n">
-        <x:v>88.247</x:v>
+        <x:v>52.184</x:v>
       </x:c>
       <x:c r="C102" s="2" t="n">
         <x:v>1</x:v>
@@ -7393,7 +7409,7 @@
         <x:v>97</x:v>
       </x:c>
       <x:c r="B103" s="8" t="n">
-        <x:v>29.975</x:v>
+        <x:v>83.769</x:v>
       </x:c>
       <x:c r="C103" s="2" t="n">
         <x:v>1</x:v>
@@ -7409,7 +7425,7 @@
         <x:v>98</x:v>
       </x:c>
       <x:c r="B104" s="8" t="n">
-        <x:v>60.793</x:v>
+        <x:v>50.559</x:v>
       </x:c>
       <x:c r="C104" s="2" t="n">
         <x:v>1</x:v>
@@ -7425,7 +7441,7 @@
         <x:v>99</x:v>
       </x:c>
       <x:c r="B105" s="8" t="n">
-        <x:v>11.4</x:v>
+        <x:v>24.677</x:v>
       </x:c>
       <x:c r="C105" s="2" t="n">
         <x:v>1</x:v>
@@ -7441,7 +7457,7 @@
         <x:v>100</x:v>
       </x:c>
       <x:c r="B106" s="8" t="n">
-        <x:v>25.829</x:v>
+        <x:v>43.27</x:v>
       </x:c>
       <x:c r="C106" s="2" t="n">
         <x:v>1</x:v>
@@ -7457,7 +7473,7 @@
         <x:v>101</x:v>
       </x:c>
       <x:c r="B107" s="8" t="n">
-        <x:v>17.069</x:v>
+        <x:v>16.244</x:v>
       </x:c>
       <x:c r="C107" s="2" t="n">
         <x:v>1</x:v>
@@ -7473,7 +7489,7 @@
         <x:v>102</x:v>
       </x:c>
       <x:c r="B108" s="8" t="n">
-        <x:v>104.518</x:v>
+        <x:v>37.268</x:v>
       </x:c>
       <x:c r="C108" s="2" t="n">
         <x:v>1</x:v>
@@ -7489,7 +7505,7 @@
         <x:v>103</x:v>
       </x:c>
       <x:c r="B109" s="8" t="n">
-        <x:v>287.754</x:v>
+        <x:v>71.666</x:v>
       </x:c>
       <x:c r="C109" s="2" t="n">
         <x:v>1</x:v>
@@ -7505,7 +7521,7 @@
         <x:v>104</x:v>
       </x:c>
       <x:c r="B110" s="8" t="n">
-        <x:v>777.011</x:v>
+        <x:v>28.755</x:v>
       </x:c>
       <x:c r="C110" s="2" t="n">
         <x:v>1</x:v>
@@ -7521,7 +7537,7 @@
         <x:v>105</x:v>
       </x:c>
       <x:c r="B111" s="8" t="n">
-        <x:v>660.821</x:v>
+        <x:v>47.139</x:v>
       </x:c>
       <x:c r="C111" s="2" t="n">
         <x:v>1</x:v>
@@ -7537,7 +7553,7 @@
         <x:v>106</x:v>
       </x:c>
       <x:c r="B112" s="8" t="n">
-        <x:v>8.073</x:v>
+        <x:v>10.632</x:v>
       </x:c>
       <x:c r="C112" s="2" t="n">
         <x:v>1</x:v>
@@ -7553,7 +7569,7 @@
         <x:v>107</x:v>
       </x:c>
       <x:c r="B113" s="8" t="n">
-        <x:v>9.232</x:v>
+        <x:v>42.098</x:v>
       </x:c>
       <x:c r="C113" s="2" t="n">
         <x:v>1</x:v>
@@ -7569,7 +7585,7 @@
         <x:v>108</x:v>
       </x:c>
       <x:c r="B114" s="8" t="n">
-        <x:v>9.744</x:v>
+        <x:v>79.914</x:v>
       </x:c>
       <x:c r="C114" s="2" t="n">
         <x:v>1</x:v>
@@ -7585,7 +7601,7 @@
         <x:v>109</x:v>
       </x:c>
       <x:c r="B115" s="8" t="n">
-        <x:v>44.779</x:v>
+        <x:v>149.351</x:v>
       </x:c>
       <x:c r="C115" s="2" t="n">
         <x:v>1</x:v>
@@ -7601,7 +7617,7 @@
         <x:v>110</x:v>
       </x:c>
       <x:c r="B116" s="8" t="n">
-        <x:v>8.658</x:v>
+        <x:v>15.616</x:v>
       </x:c>
       <x:c r="C116" s="2" t="n">
         <x:v>1</x:v>
@@ -7617,7 +7633,7 @@
         <x:v>111</x:v>
       </x:c>
       <x:c r="B117" s="8" t="n">
-        <x:v>9.806</x:v>
+        <x:v>25.826</x:v>
       </x:c>
       <x:c r="C117" s="2" t="n">
         <x:v>1</x:v>
@@ -7633,7 +7649,7 @@
         <x:v>112</x:v>
       </x:c>
       <x:c r="B118" s="8" t="n">
-        <x:v>37.305</x:v>
+        <x:v>31.019</x:v>
       </x:c>
       <x:c r="C118" s="2" t="n">
         <x:v>1</x:v>
@@ -7649,7 +7665,7 @@
         <x:v>113</x:v>
       </x:c>
       <x:c r="B119" s="8" t="n">
-        <x:v>10.646</x:v>
+        <x:v>229.854</x:v>
       </x:c>
       <x:c r="C119" s="2" t="n">
         <x:v>1</x:v>
@@ -7665,7 +7681,7 @@
         <x:v>114</x:v>
       </x:c>
       <x:c r="B120" s="8" t="n">
-        <x:v>12.538</x:v>
+        <x:v>27.232</x:v>
       </x:c>
       <x:c r="C120" s="2" t="n">
         <x:v>1</x:v>
@@ -7681,7 +7697,7 @@
         <x:v>115</x:v>
       </x:c>
       <x:c r="B121" s="8" t="n">
-        <x:v>15.449</x:v>
+        <x:v>33.249</x:v>
       </x:c>
       <x:c r="C121" s="2" t="n">
         <x:v>1</x:v>
@@ -7697,7 +7713,7 @@
         <x:v>116</x:v>
       </x:c>
       <x:c r="B122" s="8" t="n">
-        <x:v>82.504</x:v>
+        <x:v>36.591</x:v>
       </x:c>
       <x:c r="C122" s="2" t="n">
         <x:v>1</x:v>
@@ -7713,7 +7729,7 @@
         <x:v>117</x:v>
       </x:c>
       <x:c r="B123" s="8" t="n">
-        <x:v>21.243</x:v>
+        <x:v>12.793</x:v>
       </x:c>
       <x:c r="C123" s="2" t="n">
         <x:v>1</x:v>
@@ -7729,7 +7745,7 @@
         <x:v>118</x:v>
       </x:c>
       <x:c r="B124" s="8" t="n">
-        <x:v>26.512</x:v>
+        <x:v>30.783</x:v>
       </x:c>
       <x:c r="C124" s="2" t="n">
         <x:v>1</x:v>
@@ -7745,7 +7761,7 @@
         <x:v>119</x:v>
       </x:c>
       <x:c r="B125" s="8" t="n">
-        <x:v>36.918</x:v>
+        <x:v>46.852</x:v>
       </x:c>
       <x:c r="C125" s="2" t="n">
         <x:v>1</x:v>
@@ -7761,7 +7777,7 @@
         <x:v>120</x:v>
       </x:c>
       <x:c r="B126" s="8" t="n">
-        <x:v>46.727</x:v>
+        <x:v>56.03</x:v>
       </x:c>
       <x:c r="C126" s="2" t="n">
         <x:v>1</x:v>
@@ -7777,7 +7793,7 @@
         <x:v>121</x:v>
       </x:c>
       <x:c r="B127" s="8" t="n">
-        <x:v>212.828</x:v>
+        <x:v>43.737</x:v>
       </x:c>
       <x:c r="C127" s="2" t="n">
         <x:v>1</x:v>
@@ -7793,7 +7809,7 @@
         <x:v>122</x:v>
       </x:c>
       <x:c r="B128" s="8" t="n">
-        <x:v>6.982</x:v>
+        <x:v>17.522</x:v>
       </x:c>
       <x:c r="C128" s="2" t="n">
         <x:v>1</x:v>
@@ -7809,7 +7825,7 @@
         <x:v>123</x:v>
       </x:c>
       <x:c r="B129" s="8" t="n">
-        <x:v>56.717</x:v>
+        <x:v>14.484</x:v>
       </x:c>
       <x:c r="C129" s="2" t="n">
         <x:v>1</x:v>
@@ -7825,7 +7841,7 @@
         <x:v>124</x:v>
       </x:c>
       <x:c r="B130" s="8" t="n">
-        <x:v>8.57</x:v>
+        <x:v>69.019</x:v>
       </x:c>
       <x:c r="C130" s="2" t="n">
         <x:v>1</x:v>
@@ -7841,7 +7857,7 @@
         <x:v>125</x:v>
       </x:c>
       <x:c r="B131" s="8" t="n">
-        <x:v>9.344</x:v>
+        <x:v>41.65</x:v>
       </x:c>
       <x:c r="C131" s="2" t="n">
         <x:v>1</x:v>
@@ -7857,7 +7873,7 @@
         <x:v>126</x:v>
       </x:c>
       <x:c r="B132" s="8" t="n">
-        <x:v>110.478</x:v>
+        <x:v>23.054</x:v>
       </x:c>
       <x:c r="C132" s="2" t="n">
         <x:v>1</x:v>
@@ -7873,7 +7889,7 @@
         <x:v>127</x:v>
       </x:c>
       <x:c r="B133" s="8" t="n">
-        <x:v>7.989</x:v>
+        <x:v>19.283</x:v>
       </x:c>
       <x:c r="C133" s="2" t="n">
         <x:v>1</x:v>
@@ -7889,7 +7905,7 @@
         <x:v>128</x:v>
       </x:c>
       <x:c r="B134" s="8" t="n">
-        <x:v>9.525</x:v>
+        <x:v>32.863</x:v>
       </x:c>
       <x:c r="C134" s="2" t="n">
         <x:v>1</x:v>
@@ -7905,7 +7921,7 @@
         <x:v>129</x:v>
       </x:c>
       <x:c r="B135" s="8" t="n">
-        <x:v>9.125</x:v>
+        <x:v>47.751</x:v>
       </x:c>
       <x:c r="C135" s="2" t="n">
         <x:v>1</x:v>
@@ -7921,7 +7937,7 @@
         <x:v>130</x:v>
       </x:c>
       <x:c r="B136" s="8" t="n">
-        <x:v>11.166</x:v>
+        <x:v>15.748</x:v>
       </x:c>
       <x:c r="C136" s="2" t="n">
         <x:v>1</x:v>
@@ -7937,7 +7953,7 @@
         <x:v>131</x:v>
       </x:c>
       <x:c r="B137" s="8" t="n">
-        <x:v>13.756</x:v>
+        <x:v>67.283</x:v>
       </x:c>
       <x:c r="C137" s="2" t="n">
         <x:v>1</x:v>
@@ -7953,7 +7969,7 @@
         <x:v>132</x:v>
       </x:c>
       <x:c r="B138" s="8" t="n">
-        <x:v>23.399</x:v>
+        <x:v>25.637</x:v>
       </x:c>
       <x:c r="C138" s="2" t="n">
         <x:v>1</x:v>
@@ -7969,7 +7985,7 @@
         <x:v>133</x:v>
       </x:c>
       <x:c r="B139" s="8" t="n">
-        <x:v>14.79</x:v>
+        <x:v>14.232</x:v>
       </x:c>
       <x:c r="C139" s="2" t="n">
         <x:v>1</x:v>
@@ -7985,7 +8001,7 @@
         <x:v>134</x:v>
       </x:c>
       <x:c r="B140" s="8" t="n">
-        <x:v>31.265</x:v>
+        <x:v>39.042</x:v>
       </x:c>
       <x:c r="C140" s="2" t="n">
         <x:v>1</x:v>
@@ -8001,7 +8017,7 @@
         <x:v>135</x:v>
       </x:c>
       <x:c r="B141" s="8" t="n">
-        <x:v>31.458</x:v>
+        <x:v>107.748</x:v>
       </x:c>
       <x:c r="C141" s="2" t="n">
         <x:v>1</x:v>
@@ -8017,7 +8033,7 @@
         <x:v>136</x:v>
       </x:c>
       <x:c r="B142" s="8" t="n">
-        <x:v>31.659</x:v>
+        <x:v>28.649</x:v>
       </x:c>
       <x:c r="C142" s="2" t="n">
         <x:v>1</x:v>
@@ -8033,7 +8049,7 @@
         <x:v>137</x:v>
       </x:c>
       <x:c r="B143" s="8" t="n">
-        <x:v>62.218</x:v>
+        <x:v>15.065</x:v>
       </x:c>
       <x:c r="C143" s="2" t="n">
         <x:v>1</x:v>
@@ -8049,7 +8065,7 @@
         <x:v>138</x:v>
       </x:c>
       <x:c r="B144" s="8" t="n">
-        <x:v>9.581</x:v>
+        <x:v>35.834</x:v>
       </x:c>
       <x:c r="C144" s="2" t="n">
         <x:v>1</x:v>
@@ -8065,7 +8081,7 @@
         <x:v>139</x:v>
       </x:c>
       <x:c r="B145" s="8" t="n">
-        <x:v>14.852</x:v>
+        <x:v>26.376</x:v>
       </x:c>
       <x:c r="C145" s="2" t="n">
         <x:v>1</x:v>
@@ -8081,7 +8097,7 @@
         <x:v>140</x:v>
       </x:c>
       <x:c r="B146" s="8" t="n">
-        <x:v>24.385</x:v>
+        <x:v>59.466</x:v>
       </x:c>
       <x:c r="C146" s="2" t="n">
         <x:v>1</x:v>
@@ -8097,7 +8113,7 @@
         <x:v>141</x:v>
       </x:c>
       <x:c r="B147" s="8" t="n">
-        <x:v>13.911</x:v>
+        <x:v>36.107</x:v>
       </x:c>
       <x:c r="C147" s="2" t="n">
         <x:v>1</x:v>
@@ -8113,7 +8129,7 @@
         <x:v>142</x:v>
       </x:c>
       <x:c r="B148" s="8" t="n">
-        <x:v>20.359</x:v>
+        <x:v>118.921</x:v>
       </x:c>
       <x:c r="C148" s="2" t="n">
         <x:v>1</x:v>
@@ -8129,7 +8145,7 @@
         <x:v>143</x:v>
       </x:c>
       <x:c r="B149" s="8" t="n">
-        <x:v>56.642</x:v>
+        <x:v>32.508</x:v>
       </x:c>
       <x:c r="C149" s="2" t="n">
         <x:v>1</x:v>
@@ -8145,7 +8161,7 @@
         <x:v>144</x:v>
       </x:c>
       <x:c r="B150" s="8" t="n">
-        <x:v>40.364</x:v>
+        <x:v>14.544</x:v>
       </x:c>
       <x:c r="C150" s="2" t="n">
         <x:v>1</x:v>
@@ -8161,7 +8177,7 @@
         <x:v>145</x:v>
       </x:c>
       <x:c r="B151" s="8" t="n">
-        <x:v>11.669</x:v>
+        <x:v>118.758</x:v>
       </x:c>
       <x:c r="C151" s="2" t="n">
         <x:v>1</x:v>
@@ -8177,7 +8193,7 @@
         <x:v>146</x:v>
       </x:c>
       <x:c r="B152" s="8" t="n">
-        <x:v>17.153</x:v>
+        <x:v>465.17</x:v>
       </x:c>
       <x:c r="C152" s="2" t="n">
         <x:v>1</x:v>
@@ -8193,7 +8209,7 @@
         <x:v>147</x:v>
       </x:c>
       <x:c r="B153" s="8" t="n">
-        <x:v>15.704</x:v>
+        <x:v>71.356</x:v>
       </x:c>
       <x:c r="C153" s="2" t="n">
         <x:v>1</x:v>
@@ -8209,7 +8225,7 @@
         <x:v>148</x:v>
       </x:c>
       <x:c r="B154" s="8" t="n">
-        <x:v>55.581</x:v>
+        <x:v>26.683</x:v>
       </x:c>
       <x:c r="C154" s="2" t="n">
         <x:v>1</x:v>
@@ -8225,7 +8241,7 @@
         <x:v>149</x:v>
       </x:c>
       <x:c r="B155" s="8" t="n">
-        <x:v>22.585</x:v>
+        <x:v>38.753</x:v>
       </x:c>
       <x:c r="C155" s="2" t="n">
         <x:v>1</x:v>
@@ -8241,7 +8257,7 @@
         <x:v>150</x:v>
       </x:c>
       <x:c r="B156" s="8" t="n">
-        <x:v>114.849</x:v>
+        <x:v>172.542</x:v>
       </x:c>
       <x:c r="C156" s="2" t="n">
         <x:v>1</x:v>
@@ -8257,7 +8273,7 @@
         <x:v>151</x:v>
       </x:c>
       <x:c r="B157" s="8" t="n">
-        <x:v>19.023</x:v>
+        <x:v>12.954</x:v>
       </x:c>
       <x:c r="C157" s="2" t="n">
         <x:v>1</x:v>
@@ -8273,7 +8289,7 @@
         <x:v>152</x:v>
       </x:c>
       <x:c r="B158" s="8" t="n">
-        <x:v>29.013</x:v>
+        <x:v>94.931</x:v>
       </x:c>
       <x:c r="C158" s="2" t="n">
         <x:v>1</x:v>
@@ -8289,7 +8305,7 @@
         <x:v>153</x:v>
       </x:c>
       <x:c r="B159" s="8" t="n">
-        <x:v>113.846</x:v>
+        <x:v>15.865</x:v>
       </x:c>
       <x:c r="C159" s="2" t="n">
         <x:v>1</x:v>
@@ -8305,7 +8321,7 @@
         <x:v>154</x:v>
       </x:c>
       <x:c r="B160" s="8" t="n">
-        <x:v>12.322</x:v>
+        <x:v>341.722</x:v>
       </x:c>
       <x:c r="C160" s="2" t="n">
         <x:v>1</x:v>
@@ -8321,7 +8337,7 @@
         <x:v>155</x:v>
       </x:c>
       <x:c r="B161" s="8" t="n">
-        <x:v>39.876</x:v>
+        <x:v>17.527</x:v>
       </x:c>
       <x:c r="C161" s="2" t="n">
         <x:v>1</x:v>
@@ -8337,7 +8353,7 @@
         <x:v>156</x:v>
       </x:c>
       <x:c r="B162" s="8" t="n">
-        <x:v>51</x:v>
+        <x:v>47.901</x:v>
       </x:c>
       <x:c r="C162" s="2" t="n">
         <x:v>1</x:v>
@@ -8353,7 +8369,7 @@
         <x:v>157</x:v>
       </x:c>
       <x:c r="B163" s="8" t="n">
-        <x:v>32.894</x:v>
+        <x:v>14.236</x:v>
       </x:c>
       <x:c r="C163" s="2" t="n">
         <x:v>1</x:v>
@@ -8369,7 +8385,7 @@
         <x:v>158</x:v>
       </x:c>
       <x:c r="B164" s="8" t="n">
-        <x:v>15.086</x:v>
+        <x:v>18.77</x:v>
       </x:c>
       <x:c r="C164" s="2" t="n">
         <x:v>1</x:v>
@@ -8385,7 +8401,7 @@
         <x:v>159</x:v>
       </x:c>
       <x:c r="B165" s="8" t="n">
-        <x:v>14.923</x:v>
+        <x:v>35.942</x:v>
       </x:c>
       <x:c r="C165" s="2" t="n">
         <x:v>1</x:v>
@@ -8401,7 +8417,7 @@
         <x:v>160</x:v>
       </x:c>
       <x:c r="B166" s="8" t="n">
-        <x:v>46.383</x:v>
+        <x:v>110.616</x:v>
       </x:c>
       <x:c r="C166" s="2" t="n">
         <x:v>1</x:v>
@@ -8417,7 +8433,7 @@
         <x:v>161</x:v>
       </x:c>
       <x:c r="B167" s="8" t="n">
-        <x:v>11.936</x:v>
+        <x:v>9.512</x:v>
       </x:c>
       <x:c r="C167" s="2" t="n">
         <x:v>1</x:v>
@@ -8433,7 +8449,7 @@
         <x:v>162</x:v>
       </x:c>
       <x:c r="B168" s="8" t="n">
-        <x:v>14.406</x:v>
+        <x:v>11.725</x:v>
       </x:c>
       <x:c r="C168" s="2" t="n">
         <x:v>1</x:v>
@@ -8449,7 +8465,7 @@
         <x:v>163</x:v>
       </x:c>
       <x:c r="B169" s="8" t="n">
-        <x:v>17.509</x:v>
+        <x:v>63.592</x:v>
       </x:c>
       <x:c r="C169" s="2" t="n">
         <x:v>1</x:v>
@@ -8465,7 +8481,7 @@
         <x:v>164</x:v>
       </x:c>
       <x:c r="B170" s="8" t="n">
-        <x:v>151.569</x:v>
+        <x:v>13.407</x:v>
       </x:c>
       <x:c r="C170" s="2" t="n">
         <x:v>1</x:v>
@@ -8481,7 +8497,7 @@
         <x:v>165</x:v>
       </x:c>
       <x:c r="B171" s="8" t="n">
-        <x:v>67.93</x:v>
+        <x:v>16.623</x:v>
       </x:c>
       <x:c r="C171" s="2" t="n">
         <x:v>1</x:v>
@@ -8497,7 +8513,7 @@
         <x:v>166</x:v>
       </x:c>
       <x:c r="B172" s="8" t="n">
-        <x:v>11.901</x:v>
+        <x:v>30.222</x:v>
       </x:c>
       <x:c r="C172" s="2" t="n">
         <x:v>1</x:v>
@@ -8513,7 +8529,7 @@
         <x:v>167</x:v>
       </x:c>
       <x:c r="B173" s="8" t="n">
-        <x:v>260.54</x:v>
+        <x:v>17.597</x:v>
       </x:c>
       <x:c r="C173" s="2" t="n">
         <x:v>1</x:v>
@@ -8529,7 +8545,7 @@
         <x:v>168</x:v>
       </x:c>
       <x:c r="B174" s="8" t="n">
-        <x:v>9.244</x:v>
+        <x:v>29.979</x:v>
       </x:c>
       <x:c r="C174" s="2" t="n">
         <x:v>1</x:v>
@@ -8545,7 +8561,7 @@
         <x:v>169</x:v>
       </x:c>
       <x:c r="B175" s="8" t="n">
-        <x:v>13.303</x:v>
+        <x:v>13.72</x:v>
       </x:c>
       <x:c r="C175" s="2" t="n">
         <x:v>1</x:v>
@@ -8561,7 +8577,7 @@
         <x:v>170</x:v>
       </x:c>
       <x:c r="B176" s="8" t="n">
-        <x:v>32.614</x:v>
+        <x:v>35.877</x:v>
       </x:c>
       <x:c r="C176" s="2" t="n">
         <x:v>1</x:v>
@@ -8577,7 +8593,7 @@
         <x:v>171</x:v>
       </x:c>
       <x:c r="B177" s="8" t="n">
-        <x:v>9.324</x:v>
+        <x:v>15.561</x:v>
       </x:c>
       <x:c r="C177" s="2" t="n">
         <x:v>1</x:v>
@@ -8593,7 +8609,7 @@
         <x:v>172</x:v>
       </x:c>
       <x:c r="B178" s="8" t="n">
-        <x:v>122.364</x:v>
+        <x:v>13.903</x:v>
       </x:c>
       <x:c r="C178" s="2" t="n">
         <x:v>1</x:v>
@@ -8609,7 +8625,7 @@
         <x:v>173</x:v>
       </x:c>
       <x:c r="B179" s="8" t="n">
-        <x:v>31.374</x:v>
+        <x:v>27.615</x:v>
       </x:c>
       <x:c r="C179" s="2" t="n">
         <x:v>1</x:v>
@@ -8625,7 +8641,7 @@
         <x:v>174</x:v>
       </x:c>
       <x:c r="B180" s="8" t="n">
-        <x:v>76.776</x:v>
+        <x:v>56.473</x:v>
       </x:c>
       <x:c r="C180" s="2" t="n">
         <x:v>1</x:v>
@@ -8641,7 +8657,7 @@
         <x:v>175</x:v>
       </x:c>
       <x:c r="B181" s="8" t="n">
-        <x:v>24.75</x:v>
+        <x:v>34.335</x:v>
       </x:c>
       <x:c r="C181" s="2" t="n">
         <x:v>1</x:v>
@@ -8657,7 +8673,7 @@
         <x:v>176</x:v>
       </x:c>
       <x:c r="B182" s="8" t="n">
-        <x:v>45.777</x:v>
+        <x:v>22.146</x:v>
       </x:c>
       <x:c r="C182" s="2" t="n">
         <x:v>1</x:v>
@@ -8673,7 +8689,7 @@
         <x:v>177</x:v>
       </x:c>
       <x:c r="B183" s="8" t="n">
-        <x:v>10.841</x:v>
+        <x:v>45.998</x:v>
       </x:c>
       <x:c r="C183" s="2" t="n">
         <x:v>1</x:v>
@@ -8689,7 +8705,7 @@
         <x:v>178</x:v>
       </x:c>
       <x:c r="B184" s="8" t="n">
-        <x:v>14.639</x:v>
+        <x:v>43.196</x:v>
       </x:c>
       <x:c r="C184" s="2" t="n">
         <x:v>1</x:v>
@@ -8705,7 +8721,7 @@
         <x:v>179</x:v>
       </x:c>
       <x:c r="B185" s="8" t="n">
-        <x:v>8.312</x:v>
+        <x:v>45.227</x:v>
       </x:c>
       <x:c r="C185" s="2" t="n">
         <x:v>1</x:v>
@@ -8721,7 +8737,7 @@
         <x:v>180</x:v>
       </x:c>
       <x:c r="B186" s="8" t="n">
-        <x:v>11.292</x:v>
+        <x:v>13.504</x:v>
       </x:c>
       <x:c r="C186" s="2" t="n">
         <x:v>1</x:v>
@@ -8737,7 +8753,7 @@
         <x:v>181</x:v>
       </x:c>
       <x:c r="B187" s="8" t="n">
-        <x:v>13.192</x:v>
+        <x:v>12.636</x:v>
       </x:c>
       <x:c r="C187" s="2" t="n">
         <x:v>1</x:v>
@@ -8753,7 +8769,7 @@
         <x:v>182</x:v>
       </x:c>
       <x:c r="B188" s="8" t="n">
-        <x:v>15.484</x:v>
+        <x:v>149.676</x:v>
       </x:c>
       <x:c r="C188" s="2" t="n">
         <x:v>1</x:v>
@@ -8769,7 +8785,7 @@
         <x:v>183</x:v>
       </x:c>
       <x:c r="B189" s="8" t="n">
-        <x:v>26.666</x:v>
+        <x:v>65.162</x:v>
       </x:c>
       <x:c r="C189" s="2" t="n">
         <x:v>1</x:v>
@@ -8785,7 +8801,7 @@
         <x:v>184</x:v>
       </x:c>
       <x:c r="B190" s="8" t="n">
-        <x:v>11.362</x:v>
+        <x:v>23.066</x:v>
       </x:c>
       <x:c r="C190" s="2" t="n">
         <x:v>1</x:v>
@@ -8801,7 +8817,7 @@
         <x:v>185</x:v>
       </x:c>
       <x:c r="B191" s="8" t="n">
-        <x:v>10.929</x:v>
+        <x:v>27.531</x:v>
       </x:c>
       <x:c r="C191" s="2" t="n">
         <x:v>1</x:v>
@@ -8817,7 +8833,7 @@
         <x:v>186</x:v>
       </x:c>
       <x:c r="B192" s="8" t="n">
-        <x:v>65.799</x:v>
+        <x:v>159.763</x:v>
       </x:c>
       <x:c r="C192" s="2" t="n">
         <x:v>1</x:v>
@@ -8833,7 +8849,7 @@
         <x:v>187</x:v>
       </x:c>
       <x:c r="B193" s="8" t="n">
-        <x:v>76.803</x:v>
+        <x:v>61.279</x:v>
       </x:c>
       <x:c r="C193" s="2" t="n">
         <x:v>1</x:v>
@@ -8849,7 +8865,7 @@
         <x:v>188</x:v>
       </x:c>
       <x:c r="B194" s="8" t="n">
-        <x:v>14.776</x:v>
+        <x:v>14.02</x:v>
       </x:c>
       <x:c r="C194" s="2" t="n">
         <x:v>1</x:v>
@@ -8865,7 +8881,7 @@
         <x:v>189</x:v>
       </x:c>
       <x:c r="B195" s="8" t="n">
-        <x:v>113.616</x:v>
+        <x:v>14.008</x:v>
       </x:c>
       <x:c r="C195" s="2" t="n">
         <x:v>1</x:v>
@@ -8881,7 +8897,7 @@
         <x:v>190</x:v>
       </x:c>
       <x:c r="B196" s="8" t="n">
-        <x:v>31.974</x:v>
+        <x:v>14.707</x:v>
       </x:c>
       <x:c r="C196" s="2" t="n">
         <x:v>1</x:v>
@@ -8897,7 +8913,7 @@
         <x:v>191</x:v>
       </x:c>
       <x:c r="B197" s="8" t="n">
-        <x:v>7.241</x:v>
+        <x:v>12.904</x:v>
       </x:c>
       <x:c r="C197" s="2" t="n">
         <x:v>1</x:v>
@@ -8913,7 +8929,7 @@
         <x:v>192</x:v>
       </x:c>
       <x:c r="B198" s="8" t="n">
-        <x:v>9.56</x:v>
+        <x:v>11.875</x:v>
       </x:c>
       <x:c r="C198" s="2" t="n">
         <x:v>1</x:v>
@@ -8929,7 +8945,7 @@
         <x:v>193</x:v>
       </x:c>
       <x:c r="B199" s="8" t="n">
-        <x:v>27.013</x:v>
+        <x:v>11.988</x:v>
       </x:c>
       <x:c r="C199" s="2" t="n">
         <x:v>1</x:v>
@@ -8945,7 +8961,7 @@
         <x:v>194</x:v>
       </x:c>
       <x:c r="B200" s="8" t="n">
-        <x:v>8.933</x:v>
+        <x:v>54.922</x:v>
       </x:c>
       <x:c r="C200" s="2" t="n">
         <x:v>1</x:v>
@@ -8961,7 +8977,7 @@
         <x:v>195</x:v>
       </x:c>
       <x:c r="B201" s="8" t="n">
-        <x:v>8.682</x:v>
+        <x:v>19.276</x:v>
       </x:c>
       <x:c r="C201" s="2" t="n">
         <x:v>1</x:v>
@@ -8977,7 +8993,7 @@
         <x:v>196</x:v>
       </x:c>
       <x:c r="B202" s="8" t="n">
-        <x:v>45.374</x:v>
+        <x:v>41.834</x:v>
       </x:c>
       <x:c r="C202" s="2" t="n">
         <x:v>1</x:v>
@@ -8993,7 +9009,7 @@
         <x:v>197</x:v>
       </x:c>
       <x:c r="B203" s="8" t="n">
-        <x:v>15.457</x:v>
+        <x:v>15.619</x:v>
       </x:c>
       <x:c r="C203" s="2" t="n">
         <x:v>1</x:v>
@@ -9009,7 +9025,7 @@
         <x:v>198</x:v>
       </x:c>
       <x:c r="B204" s="8" t="n">
-        <x:v>25.257</x:v>
+        <x:v>16.875</x:v>
       </x:c>
       <x:c r="C204" s="2" t="n">
         <x:v>1</x:v>
@@ -9025,7 +9041,7 @@
         <x:v>199</x:v>
       </x:c>
       <x:c r="B205" s="8" t="n">
-        <x:v>13.315</x:v>
+        <x:v>14.619</x:v>
       </x:c>
       <x:c r="C205" s="2" t="n">
         <x:v>1</x:v>

</xml_diff>